<commit_message>
chore(templates): update granulometria agregados template again
</commit_message>
<xml_diff>
--- a/app/templates/informes/Informes agregado/Gran agregado AG/1-INF.-N-000-26-AG19-GRAN.-V10.xlsx
+++ b/app/templates/informes/Informes agregado/Gran agregado AG/1-INF.-N-000-26-AG19-GRAN.-V10.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lenovo\Documents\crmnew\api-geofal-crm\app\templates\informes\Informes agregado\Gran agregado AG\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{802C83FF-1FED-4BA1-B55F-38B27F5A7B59}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7E2424E-5D46-49F7-B6F0-2B47147206E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="598" firstSheet="2" activeTab="3" xr2:uid="{21CE8C7D-CFC7-4B7D-B46A-F41F71EC9170}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="598" xr2:uid="{21CE8C7D-CFC7-4B7D-B46A-F41F71EC9170}"/>
   </bookViews>
   <sheets>
     <sheet name="FORMATO" sheetId="105" r:id="rId1"/>
@@ -38418,7 +38418,7 @@
       <c r="L69" s="337"/>
     </row>
   </sheetData>
-  <sheetProtection selectLockedCells="1" selectUnlockedCells="1"/>
+  <sheetProtection sheet="1" selectLockedCells="1" selectUnlockedCells="1"/>
   <protectedRanges>
     <protectedRange sqref="E16" name="Rango3_3_1_1_1_1_1_1_1_1"/>
     <protectedRange sqref="E13" name="Rango3_3_1_1_1_1_1_1_1_1_2"/>

</xml_diff>

<commit_message>
feat(excel): validate and update gran agregado template and strip #N/A print titles
</commit_message>
<xml_diff>
--- a/app/templates/informes/Informes agregado/Gran agregado AG/1-INF.-N-000-26-AG19-GRAN.-V10.xlsx
+++ b/app/templates/informes/Informes agregado/Gran agregado AG/1-INF.-N-000-26-AG19-GRAN.-V10.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lenovo\Documents\crmnew\api-geofal-crm\app\templates\informes\Informes agregado\Gran agregado AG\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7E2424E-5D46-49F7-B6F0-2B47147206E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB5B2C2D-F79F-4238-A8AA-5D1837086A36}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="598" xr2:uid="{21CE8C7D-CFC7-4B7D-B46A-F41F71EC9170}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="598" activeTab="3" xr2:uid="{21CE8C7D-CFC7-4B7D-B46A-F41F71EC9170}"/>
   </bookViews>
   <sheets>
     <sheet name="FORMATO" sheetId="105" r:id="rId1"/>
@@ -38418,7 +38418,7 @@
       <c r="L69" s="337"/>
     </row>
   </sheetData>
-  <sheetProtection sheet="1" selectLockedCells="1" selectUnlockedCells="1"/>
+  <sheetProtection algorithmName="SHA-512" hashValue="KjtFbqj+awez3nmatvXTUhptncqa0fiqLEcNeKt9ZefP5nQ0wKPn4zyew27CVx8kYZExrWI41Hc5CswZkRF15g==" saltValue="BBTqcofuNsnULRTF5jK1Lw==" spinCount="100000" sheet="1" selectLockedCells="1" selectUnlockedCells="1"/>
   <protectedRanges>
     <protectedRange sqref="E16" name="Rango3_3_1_1_1_1_1_1_1_1"/>
     <protectedRange sqref="E13" name="Rango3_3_1_1_1_1_1_1_1_1_2"/>
@@ -38772,7 +38772,7 @@
         <v>285</v>
       </c>
       <c r="H15" s="539">
-        <f>+IF(C10="Global",FORMATO!D22,FORMATO!D36)</f>
+        <f>J12</f>
         <v>0</v>
       </c>
       <c r="I15" s="444">
@@ -40340,7 +40340,7 @@
     <row r="88" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="89" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
-  <sheetProtection sheet="1" objects="1" scenarios="1"/>
+  <sheetProtection algorithmName="SHA-512" hashValue="cvdp4ubDMsWVsh1DHGHdpbcF18q35cHVXHDDdyeqLp97E6eFY/Ur7+hm6xu3+y7OZtPYQGqOUCKbb/PsU984yw==" saltValue="HWvDGf1N7LVqZ81tzXJQUg==" spinCount="100000" sheet="1" selectLockedCells="1" selectUnlockedCells="1"/>
   <mergeCells count="15">
     <mergeCell ref="C47:E47"/>
     <mergeCell ref="C61:D61"/>
@@ -46655,7 +46655,7 @@
       <c r="I281" s="547"/>
     </row>
   </sheetData>
-  <sheetProtection sheet="1" selectLockedCells="1" selectUnlockedCells="1"/>
+  <sheetProtection algorithmName="SHA-512" hashValue="bC7OIqzPwDP9E2RGOaQfi8uGBHN1WthlXg7X1jCAP8Dds2CjtmDMblJxZi+yuB+fPcaf7Iro/t/lXx3L+YIp7A==" saltValue="oBd54LNn75iV+UT4HFB6dA==" spinCount="100000" sheet="1" selectLockedCells="1" selectUnlockedCells="1"/>
   <mergeCells count="9">
     <mergeCell ref="B280:C280"/>
     <mergeCell ref="E280:F280"/>
@@ -47898,7 +47898,7 @@
       <c r="E69" s="700"/>
     </row>
   </sheetData>
-  <sheetProtection sheet="1" selectLockedCells="1" selectUnlockedCells="1"/>
+  <sheetProtection algorithmName="SHA-512" hashValue="v8HcRHeMe336PymyxK0HQbjdnavpBQNhAw0OesYBR/orw/5sTkn/biyS02pjlqm2xZj6/AT6jSiGZpnxACuK3Q==" saltValue="8VAfBRaTo8/OhfgdVO3wyQ==" spinCount="100000" sheet="1" selectLockedCells="1" selectUnlockedCells="1"/>
   <mergeCells count="7">
     <mergeCell ref="B28:B29"/>
     <mergeCell ref="E28:E29"/>

</xml_diff>

<commit_message>
chore: update Gran Agregado template V10
</commit_message>
<xml_diff>
--- a/app/templates/informes/Informes agregado/Gran agregado AG/1-INF.-N-000-26-AG19-GRAN.-V10.xlsx
+++ b/app/templates/informes/Informes agregado/Gran agregado AG/1-INF.-N-000-26-AG19-GRAN.-V10.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lenovo\Documents\crmnew\api-geofal-crm\app\templates\informes\Informes agregado\Gran agregado AG\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E105B9FA-E8F0-4FDB-9F80-E71F3DF1F6A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F596B52-0D5A-4903-9853-7278EA5BE0CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="598" xr2:uid="{21CE8C7D-CFC7-4B7D-B46A-F41F71EC9170}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="598" activeTab="3" xr2:uid="{21CE8C7D-CFC7-4B7D-B46A-F41F71EC9170}"/>
   </bookViews>
   <sheets>
     <sheet name="FORMATO" sheetId="105" r:id="rId1"/>
@@ -6038,6 +6038,93 @@
     <xf numFmtId="0" fontId="42" fillId="7" borderId="9" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="42" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="42" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="42" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -6054,103 +6141,52 @@
       <alignment horizontal="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="177" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="178" fontId="8" fillId="0" borderId="0" xfId="11" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="166" fontId="8" fillId="0" borderId="0" xfId="11" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="42" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="42" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="42" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" wrapText="1"/>
-      <protection hidden="1"/>
+    <xf numFmtId="0" fontId="63" fillId="0" borderId="0" xfId="3" quotePrefix="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="22" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -6193,74 +6229,38 @@
       <alignment horizontal="left" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="166" fontId="8" fillId="0" borderId="0" xfId="11" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="166" fontId="8" fillId="0" borderId="22" xfId="11" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="178" fontId="8" fillId="0" borderId="0" xfId="11" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="63" fillId="0" borderId="0" xfId="3" quotePrefix="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="22" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="3" quotePrefix="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="8" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="8" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="8" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="3" quotePrefix="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="181" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="3" quotePrefix="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="8" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="8" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="8" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="3" quotePrefix="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
@@ -6419,6 +6419,46 @@
     <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="77" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="61" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
     <xf numFmtId="0" fontId="13" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection hidden="1"/>
@@ -6491,44 +6531,36 @@
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="77" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="50" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="50" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="172" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="61" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
       <protection hidden="1"/>
     </xf>
     <xf numFmtId="0" fontId="63" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1" applyProtection="1">
@@ -6549,44 +6581,6 @@
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="172" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="50" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="50" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="13" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -6604,6 +6598,9 @@
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="164" fontId="8" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
@@ -6612,6 +6609,84 @@
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection hidden="1"/>
@@ -6624,40 +6699,16 @@
       <alignment horizontal="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
       <protection hidden="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -6680,57 +6731,6 @@
     <xf numFmtId="12" fontId="12" fillId="2" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="13">
@@ -31540,34 +31540,34 @@
       <c r="M6" s="778"/>
     </row>
     <row r="7" spans="1:14" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="805" t="s">
+      <c r="A7" s="829" t="s">
         <v>2</v>
       </c>
-      <c r="B7" s="805"/>
-      <c r="C7" s="805"/>
-      <c r="D7" s="805"/>
-      <c r="E7" s="805"/>
-      <c r="F7" s="805"/>
-      <c r="G7" s="805"/>
-      <c r="H7" s="805"/>
-      <c r="I7" s="805"/>
+      <c r="B7" s="829"/>
+      <c r="C7" s="829"/>
+      <c r="D7" s="829"/>
+      <c r="E7" s="829"/>
+      <c r="F7" s="829"/>
+      <c r="G7" s="829"/>
+      <c r="H7" s="829"/>
+      <c r="I7" s="829"/>
       <c r="L7" s="285" t="s">
         <v>446</v>
       </c>
       <c r="M7" s="778"/>
     </row>
     <row r="8" spans="1:14" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="806" t="s">
+      <c r="A8" s="830" t="s">
         <v>384</v>
       </c>
-      <c r="B8" s="806"/>
-      <c r="C8" s="806"/>
-      <c r="D8" s="806"/>
-      <c r="E8" s="806"/>
-      <c r="F8" s="806"/>
-      <c r="G8" s="806"/>
-      <c r="H8" s="806"/>
-      <c r="I8" s="806"/>
+      <c r="B8" s="830"/>
+      <c r="C8" s="830"/>
+      <c r="D8" s="830"/>
+      <c r="E8" s="830"/>
+      <c r="F8" s="830"/>
+      <c r="G8" s="830"/>
+      <c r="H8" s="830"/>
+      <c r="I8" s="830"/>
       <c r="L8" s="285" t="s">
         <v>447</v>
       </c>
@@ -31590,18 +31590,18 @@
     </row>
     <row r="10" spans="1:14" ht="19.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="725"/>
-      <c r="B10" s="807" t="s">
+      <c r="B10" s="824" t="s">
         <v>385</v>
       </c>
-      <c r="C10" s="807"/>
-      <c r="D10" s="808" t="s">
+      <c r="C10" s="824"/>
+      <c r="D10" s="831" t="s">
         <v>386</v>
       </c>
-      <c r="E10" s="809"/>
-      <c r="F10" s="808" t="s">
+      <c r="E10" s="832"/>
+      <c r="F10" s="831" t="s">
         <v>387</v>
       </c>
-      <c r="G10" s="809"/>
+      <c r="G10" s="832"/>
       <c r="H10" s="736" t="s">
         <v>388</v>
       </c>
@@ -31611,12 +31611,12 @@
     </row>
     <row r="11" spans="1:14" ht="19.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="725"/>
-      <c r="B11" s="802"/>
-      <c r="C11" s="802"/>
-      <c r="D11" s="803"/>
-      <c r="E11" s="804"/>
-      <c r="F11" s="803"/>
-      <c r="G11" s="804"/>
+      <c r="B11" s="826"/>
+      <c r="C11" s="826"/>
+      <c r="D11" s="827"/>
+      <c r="E11" s="828"/>
+      <c r="F11" s="827"/>
+      <c r="G11" s="828"/>
       <c r="H11" s="737"/>
       <c r="I11" s="725"/>
       <c r="L11" s="285" t="s">
@@ -31640,17 +31640,17 @@
       <c r="M12" s="779"/>
     </row>
     <row r="13" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="811" t="s">
+      <c r="A13" s="816" t="s">
         <v>128</v>
       </c>
-      <c r="B13" s="812"/>
-      <c r="C13" s="812"/>
-      <c r="D13" s="812"/>
-      <c r="E13" s="812"/>
-      <c r="F13" s="812"/>
-      <c r="G13" s="812"/>
-      <c r="H13" s="812"/>
-      <c r="I13" s="813"/>
+      <c r="B13" s="817"/>
+      <c r="C13" s="817"/>
+      <c r="D13" s="817"/>
+      <c r="E13" s="817"/>
+      <c r="F13" s="817"/>
+      <c r="G13" s="817"/>
+      <c r="H13" s="817"/>
+      <c r="I13" s="818"/>
       <c r="J13" s="166"/>
       <c r="L13" s="285" t="s">
         <v>451</v>
@@ -31659,17 +31659,17 @@
       <c r="N13"/>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A14" s="814" t="s">
+      <c r="A14" s="819" t="s">
         <v>389</v>
       </c>
-      <c r="B14" s="815"/>
-      <c r="C14" s="815"/>
-      <c r="D14" s="815"/>
-      <c r="E14" s="815"/>
-      <c r="F14" s="815"/>
-      <c r="G14" s="815"/>
-      <c r="H14" s="815"/>
-      <c r="I14" s="816"/>
+      <c r="B14" s="820"/>
+      <c r="C14" s="820"/>
+      <c r="D14" s="820"/>
+      <c r="E14" s="820"/>
+      <c r="F14" s="820"/>
+      <c r="G14" s="820"/>
+      <c r="H14" s="820"/>
+      <c r="I14" s="821"/>
       <c r="J14" s="166"/>
       <c r="L14" s="777"/>
       <c r="M14" s="778"/>
@@ -31694,10 +31694,10 @@
       <c r="A16" s="739" t="s">
         <v>390</v>
       </c>
-      <c r="B16" s="817"/>
-      <c r="C16" s="817"/>
-      <c r="D16" s="817"/>
-      <c r="E16" s="817"/>
+      <c r="B16" s="803"/>
+      <c r="C16" s="803"/>
+      <c r="D16" s="803"/>
+      <c r="E16" s="803"/>
       <c r="F16" s="231"/>
       <c r="G16" s="213" t="s">
         <v>9</v>
@@ -31714,13 +31714,13 @@
       <c r="M16" s="780"/>
     </row>
     <row r="17" spans="1:13" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="818" t="s">
+      <c r="A17" s="822" t="s">
         <v>393</v>
       </c>
-      <c r="B17" s="818"/>
-      <c r="C17" s="818"/>
-      <c r="D17" s="819"/>
-      <c r="E17" s="819"/>
+      <c r="B17" s="822"/>
+      <c r="C17" s="822"/>
+      <c r="D17" s="823"/>
+      <c r="E17" s="823"/>
       <c r="F17" s="231"/>
       <c r="G17" s="213" t="s">
         <v>11</v>
@@ -31740,10 +31740,10 @@
       <c r="A18" s="739" t="s">
         <v>396</v>
       </c>
-      <c r="B18" s="817"/>
-      <c r="C18" s="817"/>
-      <c r="D18" s="817"/>
-      <c r="E18" s="817"/>
+      <c r="B18" s="803"/>
+      <c r="C18" s="803"/>
+      <c r="D18" s="803"/>
+      <c r="E18" s="803"/>
       <c r="F18" s="740"/>
       <c r="G18" s="77" t="s">
         <v>397</v>
@@ -31765,13 +31765,13 @@
       <c r="I19" s="69"/>
     </row>
     <row r="20" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="807" t="s">
+      <c r="A20" s="824" t="s">
         <v>399</v>
       </c>
-      <c r="B20" s="807"/>
-      <c r="C20" s="807"/>
-      <c r="D20" s="807"/>
-      <c r="E20" s="807"/>
+      <c r="B20" s="824"/>
+      <c r="C20" s="824"/>
+      <c r="D20" s="824"/>
+      <c r="E20" s="824"/>
       <c r="F20" s="742"/>
       <c r="G20" s="77" t="s">
         <v>400</v>
@@ -31790,8 +31790,8 @@
       <c r="C21" s="745" t="s">
         <v>402</v>
       </c>
-      <c r="D21" s="820"/>
-      <c r="E21" s="820"/>
+      <c r="D21" s="825"/>
+      <c r="E21" s="825"/>
       <c r="F21" s="746"/>
       <c r="G21" s="77" t="s">
         <v>403</v>
@@ -31810,8 +31810,8 @@
       <c r="C22" s="745" t="s">
         <v>402</v>
       </c>
-      <c r="D22" s="820"/>
-      <c r="E22" s="820"/>
+      <c r="D22" s="825"/>
+      <c r="E22" s="825"/>
       <c r="F22" s="746"/>
       <c r="G22" s="77" t="s">
         <v>405</v>
@@ -31829,8 +31829,8 @@
       <c r="C23" s="745" t="s">
         <v>402</v>
       </c>
-      <c r="D23" s="820"/>
-      <c r="E23" s="820"/>
+      <c r="D23" s="825"/>
+      <c r="E23" s="825"/>
       <c r="F23" s="746"/>
       <c r="G23" s="77" t="s">
         <v>407</v>
@@ -31848,8 +31848,8 @@
       <c r="C24" s="745" t="s">
         <v>402</v>
       </c>
-      <c r="D24" s="820"/>
-      <c r="E24" s="820"/>
+      <c r="D24" s="825"/>
+      <c r="E24" s="825"/>
       <c r="F24" s="746"/>
       <c r="G24" s="220" t="s">
         <v>409</v>
@@ -31875,13 +31875,13 @@
       <c r="I25" s="69"/>
     </row>
     <row r="26" spans="1:13" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="810" t="s">
+      <c r="A26" s="815" t="s">
         <v>411</v>
       </c>
-      <c r="B26" s="810"/>
-      <c r="C26" s="810"/>
-      <c r="D26" s="810"/>
-      <c r="E26" s="810"/>
+      <c r="B26" s="815"/>
+      <c r="C26" s="815"/>
+      <c r="D26" s="815"/>
+      <c r="E26" s="815"/>
       <c r="F26" s="5"/>
       <c r="G26" s="77" t="s">
         <v>412</v>
@@ -31899,8 +31899,8 @@
       <c r="C27" s="750" t="s">
         <v>402</v>
       </c>
-      <c r="D27" s="821"/>
-      <c r="E27" s="821"/>
+      <c r="D27" s="811"/>
+      <c r="E27" s="811"/>
       <c r="G27" s="220" t="s">
         <v>413</v>
       </c>
@@ -31917,8 +31917,8 @@
       <c r="C28" s="752" t="s">
         <v>402</v>
       </c>
-      <c r="D28" s="817"/>
-      <c r="E28" s="817"/>
+      <c r="D28" s="803"/>
+      <c r="E28" s="803"/>
       <c r="G28" s="77" t="s">
         <v>415</v>
       </c>
@@ -31928,13 +31928,13 @@
       <c r="I28" s="69"/>
     </row>
     <row r="29" spans="1:13" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="822" t="s">
+      <c r="A29" s="812" t="s">
         <v>416</v>
       </c>
-      <c r="B29" s="823"/>
-      <c r="C29" s="823"/>
-      <c r="D29" s="823"/>
-      <c r="E29" s="824"/>
+      <c r="B29" s="813"/>
+      <c r="C29" s="813"/>
+      <c r="D29" s="813"/>
+      <c r="E29" s="814"/>
       <c r="G29" s="220" t="s">
         <v>417</v>
       </c>
@@ -31952,8 +31952,8 @@
       <c r="C30" s="752" t="s">
         <v>402</v>
       </c>
-      <c r="D30" s="817"/>
-      <c r="E30" s="817"/>
+      <c r="D30" s="803"/>
+      <c r="E30" s="803"/>
       <c r="G30" s="220" t="s">
         <v>161</v>
       </c>
@@ -31971,8 +31971,8 @@
       <c r="C31" s="752" t="s">
         <v>402</v>
       </c>
-      <c r="D31" s="817"/>
-      <c r="E31" s="817"/>
+      <c r="D31" s="803"/>
+      <c r="E31" s="803"/>
       <c r="G31" s="220" t="s">
         <v>418</v>
       </c>
@@ -31983,13 +31983,13 @@
       <c r="J31" s="166"/>
     </row>
     <row r="32" spans="1:13" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="822" t="s">
+      <c r="A32" s="812" t="s">
         <v>419</v>
       </c>
-      <c r="B32" s="823"/>
-      <c r="C32" s="823"/>
-      <c r="D32" s="823"/>
-      <c r="E32" s="824"/>
+      <c r="B32" s="813"/>
+      <c r="C32" s="813"/>
+      <c r="D32" s="813"/>
+      <c r="E32" s="814"/>
       <c r="G32" s="220" t="s">
         <v>420</v>
       </c>
@@ -32007,8 +32007,8 @@
       <c r="C33" s="752" t="s">
         <v>402</v>
       </c>
-      <c r="D33" s="817"/>
-      <c r="E33" s="817"/>
+      <c r="D33" s="803"/>
+      <c r="E33" s="803"/>
       <c r="F33" s="740"/>
       <c r="G33" s="220" t="s">
         <v>422</v>
@@ -32026,8 +32026,8 @@
       <c r="C34" s="747" t="s">
         <v>402</v>
       </c>
-      <c r="D34" s="817"/>
-      <c r="E34" s="817"/>
+      <c r="D34" s="803"/>
+      <c r="E34" s="803"/>
       <c r="F34" s="740"/>
       <c r="G34" s="220" t="s">
         <v>424</v>
@@ -32046,8 +32046,8 @@
       <c r="C35" s="752" t="s">
         <v>402</v>
       </c>
-      <c r="D35" s="817"/>
-      <c r="E35" s="817"/>
+      <c r="D35" s="803"/>
+      <c r="E35" s="803"/>
       <c r="F35" s="740"/>
       <c r="G35" s="230" t="s">
         <v>34</v>
@@ -32065,8 +32065,8 @@
       <c r="C36" s="747" t="s">
         <v>402</v>
       </c>
-      <c r="D36" s="817"/>
-      <c r="E36" s="817"/>
+      <c r="D36" s="803"/>
+      <c r="E36" s="803"/>
       <c r="F36" s="740"/>
       <c r="H36" s="755" t="s">
         <v>427</v>
@@ -32081,8 +32081,8 @@
       <c r="C37" s="752" t="s">
         <v>402</v>
       </c>
-      <c r="D37" s="817"/>
-      <c r="E37" s="817"/>
+      <c r="D37" s="803"/>
+      <c r="E37" s="803"/>
       <c r="F37" s="740"/>
       <c r="J37" s="166"/>
     </row>
@@ -32094,8 +32094,8 @@
       <c r="C38" s="750" t="s">
         <v>430</v>
       </c>
-      <c r="D38" s="817"/>
-      <c r="E38" s="817"/>
+      <c r="D38" s="803"/>
+      <c r="E38" s="803"/>
       <c r="F38" s="740"/>
       <c r="I38" s="757"/>
       <c r="J38" s="166"/>
@@ -32108,8 +32108,8 @@
       <c r="C39" s="750" t="s">
         <v>402</v>
       </c>
-      <c r="D39" s="817"/>
-      <c r="E39" s="817"/>
+      <c r="D39" s="803"/>
+      <c r="E39" s="803"/>
       <c r="F39" s="740"/>
       <c r="G39" s="758"/>
       <c r="H39" s="759"/>
@@ -32125,12 +32125,12 @@
       <c r="J40" s="166"/>
     </row>
     <row r="41" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="826" t="s">
+      <c r="A41" s="804" t="s">
         <v>432</v>
       </c>
-      <c r="B41" s="826"/>
-      <c r="C41" s="826"/>
-      <c r="D41" s="826"/>
+      <c r="B41" s="804"/>
+      <c r="C41" s="804"/>
+      <c r="D41" s="804"/>
       <c r="E41" s="760"/>
       <c r="F41" s="760"/>
       <c r="J41" s="166"/>
@@ -32140,10 +32140,10 @@
         <v>433</v>
       </c>
       <c r="B42" s="762"/>
-      <c r="C42" s="827"/>
-      <c r="D42" s="827"/>
-      <c r="E42" s="828"/>
-      <c r="F42" s="828"/>
+      <c r="C42" s="805"/>
+      <c r="D42" s="805"/>
+      <c r="E42" s="806"/>
+      <c r="F42" s="806"/>
       <c r="J42" s="166"/>
     </row>
     <row r="43" spans="1:10" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -32151,10 +32151,10 @@
         <v>434</v>
       </c>
       <c r="B43" s="763"/>
-      <c r="C43" s="827"/>
-      <c r="D43" s="827"/>
-      <c r="E43" s="828"/>
-      <c r="F43" s="828"/>
+      <c r="C43" s="805"/>
+      <c r="D43" s="805"/>
+      <c r="E43" s="806"/>
+      <c r="F43" s="806"/>
       <c r="J43" s="166"/>
     </row>
     <row r="44" spans="1:10" ht="21" customHeight="1" x14ac:dyDescent="0.25">
@@ -32162,10 +32162,10 @@
         <v>435</v>
       </c>
       <c r="B44" s="763"/>
-      <c r="C44" s="827"/>
-      <c r="D44" s="827"/>
-      <c r="E44" s="828"/>
-      <c r="F44" s="828"/>
+      <c r="C44" s="805"/>
+      <c r="D44" s="805"/>
+      <c r="E44" s="806"/>
+      <c r="F44" s="806"/>
       <c r="J44" s="166"/>
     </row>
     <row r="45" spans="1:10" ht="6.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -32188,25 +32188,25 @@
       <c r="A47" s="769" t="s">
         <v>438</v>
       </c>
-      <c r="B47" s="829"/>
-      <c r="C47" s="830"/>
-      <c r="D47" s="831"/>
+      <c r="B47" s="807"/>
+      <c r="C47" s="808"/>
+      <c r="D47" s="809"/>
       <c r="E47" s="247"/>
       <c r="F47" s="247"/>
-      <c r="G47" s="832" t="s">
+      <c r="G47" s="810" t="s">
         <v>439</v>
       </c>
-      <c r="H47" s="832"/>
-      <c r="I47" s="832"/>
+      <c r="H47" s="810"/>
+      <c r="I47" s="810"/>
       <c r="J47" s="166"/>
     </row>
     <row r="48" spans="1:10" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="770" t="s">
         <v>440</v>
       </c>
-      <c r="B48" s="829"/>
-      <c r="C48" s="830"/>
-      <c r="D48" s="831"/>
+      <c r="B48" s="807"/>
+      <c r="C48" s="808"/>
+      <c r="D48" s="809"/>
       <c r="E48" s="247"/>
       <c r="F48" s="247"/>
       <c r="G48" s="4" t="s">
@@ -32271,17 +32271,17 @@
     </row>
     <row r="54" spans="1:10" ht="3.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="55" spans="1:10" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A55" s="825" t="s">
+      <c r="A55" s="802" t="s">
         <v>445</v>
       </c>
-      <c r="B55" s="825"/>
-      <c r="C55" s="825"/>
-      <c r="D55" s="825"/>
-      <c r="E55" s="825"/>
-      <c r="F55" s="825"/>
-      <c r="G55" s="825"/>
-      <c r="H55" s="825"/>
-      <c r="I55" s="825"/>
+      <c r="B55" s="802"/>
+      <c r="C55" s="802"/>
+      <c r="D55" s="802"/>
+      <c r="E55" s="802"/>
+      <c r="F55" s="802"/>
+      <c r="G55" s="802"/>
+      <c r="H55" s="802"/>
+      <c r="I55" s="802"/>
     </row>
     <row r="56" spans="1:10" ht="15.9" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="57" spans="1:10" ht="15.9" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -32291,6 +32291,38 @@
     <protectedRange sqref="B15" name="Rango3_3_1_1_1_1_1_1_1_1"/>
   </protectedRanges>
   <mergeCells count="44">
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="D11:E11"/>
+    <mergeCell ref="F11:G11"/>
+    <mergeCell ref="A7:I7"/>
+    <mergeCell ref="A8:I8"/>
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="D10:E10"/>
+    <mergeCell ref="F10:G10"/>
+    <mergeCell ref="A26:E26"/>
+    <mergeCell ref="A13:I13"/>
+    <mergeCell ref="A14:I14"/>
+    <mergeCell ref="B16:E16"/>
+    <mergeCell ref="A17:C17"/>
+    <mergeCell ref="D17:E17"/>
+    <mergeCell ref="B18:E18"/>
+    <mergeCell ref="A20:E20"/>
+    <mergeCell ref="D21:E21"/>
+    <mergeCell ref="D22:E22"/>
+    <mergeCell ref="D23:E23"/>
+    <mergeCell ref="D24:E24"/>
+    <mergeCell ref="D38:E38"/>
+    <mergeCell ref="D27:E27"/>
+    <mergeCell ref="D28:E28"/>
+    <mergeCell ref="A29:E29"/>
+    <mergeCell ref="D30:E30"/>
+    <mergeCell ref="D31:E31"/>
+    <mergeCell ref="A32:E32"/>
+    <mergeCell ref="D33:E33"/>
+    <mergeCell ref="D34:E34"/>
+    <mergeCell ref="D35:E35"/>
+    <mergeCell ref="D36:E36"/>
+    <mergeCell ref="D37:E37"/>
     <mergeCell ref="A55:I55"/>
     <mergeCell ref="D39:E39"/>
     <mergeCell ref="A41:D41"/>
@@ -32303,38 +32335,6 @@
     <mergeCell ref="B47:D47"/>
     <mergeCell ref="G47:I47"/>
     <mergeCell ref="B48:D48"/>
-    <mergeCell ref="D38:E38"/>
-    <mergeCell ref="D27:E27"/>
-    <mergeCell ref="D28:E28"/>
-    <mergeCell ref="A29:E29"/>
-    <mergeCell ref="D30:E30"/>
-    <mergeCell ref="D31:E31"/>
-    <mergeCell ref="A32:E32"/>
-    <mergeCell ref="D33:E33"/>
-    <mergeCell ref="D34:E34"/>
-    <mergeCell ref="D35:E35"/>
-    <mergeCell ref="D36:E36"/>
-    <mergeCell ref="D37:E37"/>
-    <mergeCell ref="A26:E26"/>
-    <mergeCell ref="A13:I13"/>
-    <mergeCell ref="A14:I14"/>
-    <mergeCell ref="B16:E16"/>
-    <mergeCell ref="A17:C17"/>
-    <mergeCell ref="D17:E17"/>
-    <mergeCell ref="B18:E18"/>
-    <mergeCell ref="A20:E20"/>
-    <mergeCell ref="D21:E21"/>
-    <mergeCell ref="D22:E22"/>
-    <mergeCell ref="D23:E23"/>
-    <mergeCell ref="D24:E24"/>
-    <mergeCell ref="B11:C11"/>
-    <mergeCell ref="D11:E11"/>
-    <mergeCell ref="F11:G11"/>
-    <mergeCell ref="A7:I7"/>
-    <mergeCell ref="A8:I8"/>
-    <mergeCell ref="B10:C10"/>
-    <mergeCell ref="D10:E10"/>
-    <mergeCell ref="F10:G10"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0" right="0.59055118110236227" top="0.78740157480314965" bottom="0" header="0" footer="0"/>
@@ -32387,117 +32387,117 @@
       <c r="T4" s="25"/>
     </row>
     <row r="5" spans="2:55" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B5" s="974" t="s">
+      <c r="B5" s="995" t="s">
         <v>67</v>
       </c>
-      <c r="C5" s="975"/>
-      <c r="D5" s="975"/>
-      <c r="E5" s="975"/>
-      <c r="F5" s="976"/>
-      <c r="H5" s="974" t="s">
+      <c r="C5" s="996"/>
+      <c r="D5" s="996"/>
+      <c r="E5" s="996"/>
+      <c r="F5" s="997"/>
+      <c r="H5" s="995" t="s">
         <v>67</v>
       </c>
-      <c r="I5" s="975"/>
-      <c r="J5" s="975"/>
-      <c r="K5" s="975"/>
-      <c r="L5" s="975"/>
-      <c r="M5" s="975"/>
-      <c r="N5" s="975"/>
-      <c r="O5" s="975"/>
-      <c r="P5" s="975"/>
-      <c r="Q5" s="975"/>
-      <c r="R5" s="975"/>
-      <c r="S5" s="975"/>
-      <c r="T5" s="975"/>
-      <c r="U5" s="975"/>
-      <c r="V5" s="975"/>
-      <c r="W5" s="975"/>
-      <c r="X5" s="975"/>
-      <c r="Y5" s="975"/>
-      <c r="Z5" s="975"/>
-      <c r="AA5" s="975"/>
-      <c r="AB5" s="975"/>
-      <c r="AC5" s="975"/>
-      <c r="AD5" s="975"/>
-      <c r="AE5" s="975"/>
-      <c r="AF5" s="975"/>
-      <c r="AG5" s="975"/>
-      <c r="AH5" s="975"/>
-      <c r="AI5" s="975"/>
-      <c r="AJ5" s="975"/>
-      <c r="AK5" s="975"/>
-      <c r="AL5" s="975"/>
-      <c r="AM5" s="975"/>
-      <c r="AN5" s="975"/>
-      <c r="AO5" s="975"/>
-      <c r="AP5" s="975"/>
-      <c r="AQ5" s="975"/>
-      <c r="AR5" s="975"/>
-      <c r="AS5" s="976"/>
+      <c r="I5" s="996"/>
+      <c r="J5" s="996"/>
+      <c r="K5" s="996"/>
+      <c r="L5" s="996"/>
+      <c r="M5" s="996"/>
+      <c r="N5" s="996"/>
+      <c r="O5" s="996"/>
+      <c r="P5" s="996"/>
+      <c r="Q5" s="996"/>
+      <c r="R5" s="996"/>
+      <c r="S5" s="996"/>
+      <c r="T5" s="996"/>
+      <c r="U5" s="996"/>
+      <c r="V5" s="996"/>
+      <c r="W5" s="996"/>
+      <c r="X5" s="996"/>
+      <c r="Y5" s="996"/>
+      <c r="Z5" s="996"/>
+      <c r="AA5" s="996"/>
+      <c r="AB5" s="996"/>
+      <c r="AC5" s="996"/>
+      <c r="AD5" s="996"/>
+      <c r="AE5" s="996"/>
+      <c r="AF5" s="996"/>
+      <c r="AG5" s="996"/>
+      <c r="AH5" s="996"/>
+      <c r="AI5" s="996"/>
+      <c r="AJ5" s="996"/>
+      <c r="AK5" s="996"/>
+      <c r="AL5" s="996"/>
+      <c r="AM5" s="996"/>
+      <c r="AN5" s="996"/>
+      <c r="AO5" s="996"/>
+      <c r="AP5" s="996"/>
+      <c r="AQ5" s="996"/>
+      <c r="AR5" s="996"/>
+      <c r="AS5" s="997"/>
     </row>
     <row r="6" spans="2:55" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B6" s="974" t="s">
+      <c r="B6" s="995" t="s">
         <v>66</v>
       </c>
-      <c r="C6" s="975"/>
-      <c r="D6" s="975"/>
-      <c r="E6" s="975"/>
-      <c r="F6" s="976"/>
-      <c r="H6" s="974" t="s">
+      <c r="C6" s="996"/>
+      <c r="D6" s="996"/>
+      <c r="E6" s="996"/>
+      <c r="F6" s="997"/>
+      <c r="H6" s="995" t="s">
         <v>68</v>
       </c>
-      <c r="I6" s="975"/>
-      <c r="J6" s="975"/>
-      <c r="K6" s="975"/>
-      <c r="L6" s="975"/>
-      <c r="M6" s="975"/>
-      <c r="N6" s="975"/>
-      <c r="O6" s="975"/>
-      <c r="P6" s="975"/>
-      <c r="Q6" s="975"/>
-      <c r="R6" s="975"/>
-      <c r="S6" s="975"/>
-      <c r="T6" s="975"/>
-      <c r="U6" s="975"/>
-      <c r="V6" s="975"/>
-      <c r="W6" s="975"/>
-      <c r="X6" s="975"/>
-      <c r="Y6" s="975"/>
-      <c r="Z6" s="975"/>
-      <c r="AA6" s="975"/>
-      <c r="AB6" s="975"/>
-      <c r="AC6" s="975"/>
-      <c r="AD6" s="975"/>
-      <c r="AE6" s="975"/>
-      <c r="AF6" s="975"/>
-      <c r="AG6" s="975"/>
-      <c r="AH6" s="975"/>
-      <c r="AI6" s="975"/>
-      <c r="AJ6" s="975"/>
-      <c r="AK6" s="975"/>
-      <c r="AL6" s="975"/>
-      <c r="AM6" s="975"/>
-      <c r="AN6" s="975"/>
-      <c r="AO6" s="975"/>
-      <c r="AP6" s="975"/>
-      <c r="AQ6" s="975"/>
-      <c r="AR6" s="975"/>
-      <c r="AS6" s="976"/>
+      <c r="I6" s="996"/>
+      <c r="J6" s="996"/>
+      <c r="K6" s="996"/>
+      <c r="L6" s="996"/>
+      <c r="M6" s="996"/>
+      <c r="N6" s="996"/>
+      <c r="O6" s="996"/>
+      <c r="P6" s="996"/>
+      <c r="Q6" s="996"/>
+      <c r="R6" s="996"/>
+      <c r="S6" s="996"/>
+      <c r="T6" s="996"/>
+      <c r="U6" s="996"/>
+      <c r="V6" s="996"/>
+      <c r="W6" s="996"/>
+      <c r="X6" s="996"/>
+      <c r="Y6" s="996"/>
+      <c r="Z6" s="996"/>
+      <c r="AA6" s="996"/>
+      <c r="AB6" s="996"/>
+      <c r="AC6" s="996"/>
+      <c r="AD6" s="996"/>
+      <c r="AE6" s="996"/>
+      <c r="AF6" s="996"/>
+      <c r="AG6" s="996"/>
+      <c r="AH6" s="996"/>
+      <c r="AI6" s="996"/>
+      <c r="AJ6" s="996"/>
+      <c r="AK6" s="996"/>
+      <c r="AL6" s="996"/>
+      <c r="AM6" s="996"/>
+      <c r="AN6" s="996"/>
+      <c r="AO6" s="996"/>
+      <c r="AP6" s="996"/>
+      <c r="AQ6" s="996"/>
+      <c r="AR6" s="996"/>
+      <c r="AS6" s="997"/>
     </row>
     <row r="7" spans="2:55" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B7" s="999" t="s">
+      <c r="B7" s="975" t="s">
         <v>9</v>
       </c>
-      <c r="C7" s="1000"/>
-      <c r="D7" s="977" t="s">
+      <c r="C7" s="976"/>
+      <c r="D7" s="979" t="s">
         <v>46</v>
       </c>
-      <c r="E7" s="978"/>
-      <c r="F7" s="979"/>
-      <c r="H7" s="1003" t="s">
+      <c r="E7" s="980"/>
+      <c r="F7" s="981"/>
+      <c r="H7" s="991" t="s">
         <v>65</v>
       </c>
-      <c r="I7" s="1004"/>
+      <c r="I7" s="992"/>
       <c r="J7" s="30"/>
       <c r="K7" s="30"/>
       <c r="L7" s="30"/>
@@ -32507,119 +32507,119 @@
       <c r="P7" s="30"/>
       <c r="Q7" s="30"/>
       <c r="R7" s="14"/>
-      <c r="S7" s="989">
+      <c r="S7" s="1004">
         <v>2</v>
       </c>
-      <c r="T7" s="990"/>
-      <c r="U7" s="991"/>
-      <c r="V7" s="995"/>
-      <c r="W7" s="996"/>
-      <c r="X7" s="997"/>
-      <c r="Y7" s="989">
+      <c r="T7" s="1005"/>
+      <c r="U7" s="1006"/>
+      <c r="V7" s="998"/>
+      <c r="W7" s="999"/>
+      <c r="X7" s="1000"/>
+      <c r="Y7" s="1004">
         <v>1.5</v>
       </c>
-      <c r="Z7" s="990"/>
-      <c r="AA7" s="991"/>
-      <c r="AB7" s="995"/>
-      <c r="AC7" s="996"/>
-      <c r="AD7" s="997"/>
-      <c r="AE7" s="995"/>
-      <c r="AF7" s="996"/>
-      <c r="AG7" s="997"/>
-      <c r="AH7" s="989">
+      <c r="Z7" s="1005"/>
+      <c r="AA7" s="1006"/>
+      <c r="AB7" s="998"/>
+      <c r="AC7" s="999"/>
+      <c r="AD7" s="1000"/>
+      <c r="AE7" s="998"/>
+      <c r="AF7" s="999"/>
+      <c r="AG7" s="1000"/>
+      <c r="AH7" s="1004">
         <v>1</v>
       </c>
-      <c r="AI7" s="990"/>
-      <c r="AJ7" s="991"/>
-      <c r="AK7" s="995"/>
-      <c r="AL7" s="996"/>
-      <c r="AM7" s="997"/>
-      <c r="AN7" s="989">
+      <c r="AI7" s="1005"/>
+      <c r="AJ7" s="1006"/>
+      <c r="AK7" s="998"/>
+      <c r="AL7" s="999"/>
+      <c r="AM7" s="1000"/>
+      <c r="AN7" s="1004">
         <v>0.75</v>
       </c>
-      <c r="AO7" s="990"/>
-      <c r="AP7" s="991"/>
-      <c r="AQ7" s="989">
+      <c r="AO7" s="1005"/>
+      <c r="AP7" s="1006"/>
+      <c r="AQ7" s="1004">
         <v>0.5</v>
       </c>
-      <c r="AR7" s="990"/>
-      <c r="AS7" s="991"/>
+      <c r="AR7" s="1005"/>
+      <c r="AS7" s="1006"/>
     </row>
     <row r="8" spans="2:55" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B8" s="1001"/>
-      <c r="C8" s="1002"/>
-      <c r="D8" s="980"/>
-      <c r="E8" s="981"/>
-      <c r="F8" s="982"/>
-      <c r="H8" s="1005" t="s">
+      <c r="B8" s="977"/>
+      <c r="C8" s="978"/>
+      <c r="D8" s="982"/>
+      <c r="E8" s="983"/>
+      <c r="F8" s="984"/>
+      <c r="H8" s="993" t="s">
         <v>64</v>
       </c>
-      <c r="I8" s="1006"/>
-      <c r="J8" s="992">
+      <c r="I8" s="994"/>
+      <c r="J8" s="988">
         <v>1</v>
       </c>
-      <c r="K8" s="993"/>
-      <c r="L8" s="994"/>
-      <c r="M8" s="992">
+      <c r="K8" s="989"/>
+      <c r="L8" s="990"/>
+      <c r="M8" s="988">
         <v>2</v>
       </c>
-      <c r="N8" s="993"/>
-      <c r="O8" s="994"/>
-      <c r="P8" s="992">
+      <c r="N8" s="989"/>
+      <c r="O8" s="990"/>
+      <c r="P8" s="988">
         <v>3</v>
       </c>
-      <c r="Q8" s="993"/>
-      <c r="R8" s="994"/>
-      <c r="S8" s="992">
+      <c r="Q8" s="989"/>
+      <c r="R8" s="990"/>
+      <c r="S8" s="988">
         <v>357</v>
       </c>
-      <c r="T8" s="993"/>
-      <c r="U8" s="994"/>
-      <c r="V8" s="992">
+      <c r="T8" s="989"/>
+      <c r="U8" s="990"/>
+      <c r="V8" s="988">
         <v>4</v>
       </c>
-      <c r="W8" s="993"/>
-      <c r="X8" s="994"/>
-      <c r="Y8" s="992">
+      <c r="W8" s="989"/>
+      <c r="X8" s="990"/>
+      <c r="Y8" s="988">
         <v>467</v>
       </c>
-      <c r="Z8" s="993"/>
-      <c r="AA8" s="994"/>
-      <c r="AB8" s="992">
+      <c r="Z8" s="989"/>
+      <c r="AA8" s="990"/>
+      <c r="AB8" s="988">
         <v>5</v>
       </c>
-      <c r="AC8" s="993"/>
-      <c r="AD8" s="994"/>
-      <c r="AE8" s="992">
+      <c r="AC8" s="989"/>
+      <c r="AD8" s="990"/>
+      <c r="AE8" s="988">
         <v>56</v>
       </c>
-      <c r="AF8" s="993"/>
-      <c r="AG8" s="994"/>
-      <c r="AH8" s="992">
+      <c r="AF8" s="989"/>
+      <c r="AG8" s="990"/>
+      <c r="AH8" s="988">
         <v>57</v>
       </c>
-      <c r="AI8" s="993"/>
-      <c r="AJ8" s="994"/>
-      <c r="AK8" s="992">
+      <c r="AI8" s="989"/>
+      <c r="AJ8" s="990"/>
+      <c r="AK8" s="988">
         <v>6</v>
       </c>
-      <c r="AL8" s="993"/>
-      <c r="AM8" s="994"/>
-      <c r="AN8" s="992">
+      <c r="AL8" s="989"/>
+      <c r="AM8" s="990"/>
+      <c r="AN8" s="988">
         <v>67</v>
       </c>
-      <c r="AO8" s="993"/>
-      <c r="AP8" s="994"/>
-      <c r="AQ8" s="992">
+      <c r="AO8" s="989"/>
+      <c r="AP8" s="990"/>
+      <c r="AQ8" s="988">
         <v>7</v>
       </c>
-      <c r="AR8" s="993"/>
-      <c r="AS8" s="994"/>
-      <c r="AT8" s="992">
+      <c r="AR8" s="989"/>
+      <c r="AS8" s="990"/>
+      <c r="AT8" s="988">
         <v>8</v>
       </c>
-      <c r="AU8" s="993"/>
-      <c r="AV8" s="994"/>
+      <c r="AU8" s="989"/>
+      <c r="AV8" s="990"/>
     </row>
     <row r="9" spans="2:55" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B9" s="31" t="s">
@@ -32628,80 +32628,80 @@
       <c r="C9" s="31" t="s">
         <v>12</v>
       </c>
-      <c r="D9" s="983"/>
-      <c r="E9" s="984"/>
-      <c r="F9" s="985"/>
+      <c r="D9" s="985"/>
+      <c r="E9" s="986"/>
+      <c r="F9" s="987"/>
       <c r="H9" s="32" t="s">
         <v>11</v>
       </c>
       <c r="I9" s="32" t="s">
         <v>12</v>
       </c>
-      <c r="J9" s="992" t="s">
+      <c r="J9" s="988" t="s">
         <v>51</v>
       </c>
-      <c r="K9" s="993"/>
-      <c r="L9" s="994"/>
-      <c r="M9" s="992" t="s">
+      <c r="K9" s="989"/>
+      <c r="L9" s="990"/>
+      <c r="M9" s="988" t="s">
         <v>52</v>
       </c>
-      <c r="N9" s="993"/>
-      <c r="O9" s="994"/>
-      <c r="P9" s="992" t="s">
+      <c r="N9" s="989"/>
+      <c r="O9" s="990"/>
+      <c r="P9" s="988" t="s">
         <v>53</v>
       </c>
-      <c r="Q9" s="993"/>
-      <c r="R9" s="994"/>
-      <c r="S9" s="992" t="s">
+      <c r="Q9" s="989"/>
+      <c r="R9" s="990"/>
+      <c r="S9" s="988" t="s">
         <v>54</v>
       </c>
-      <c r="T9" s="993"/>
-      <c r="U9" s="994"/>
-      <c r="V9" s="992" t="s">
+      <c r="T9" s="989"/>
+      <c r="U9" s="990"/>
+      <c r="V9" s="988" t="s">
         <v>55</v>
       </c>
-      <c r="W9" s="993"/>
-      <c r="X9" s="994"/>
-      <c r="Y9" s="992" t="s">
+      <c r="W9" s="989"/>
+      <c r="X9" s="990"/>
+      <c r="Y9" s="988" t="s">
         <v>56</v>
       </c>
-      <c r="Z9" s="993"/>
-      <c r="AA9" s="994"/>
-      <c r="AB9" s="992" t="s">
+      <c r="Z9" s="989"/>
+      <c r="AA9" s="990"/>
+      <c r="AB9" s="988" t="s">
         <v>57</v>
       </c>
-      <c r="AC9" s="993"/>
-      <c r="AD9" s="994"/>
-      <c r="AE9" s="992" t="s">
+      <c r="AC9" s="989"/>
+      <c r="AD9" s="990"/>
+      <c r="AE9" s="988" t="s">
         <v>58</v>
       </c>
-      <c r="AF9" s="993"/>
-      <c r="AG9" s="994"/>
-      <c r="AH9" s="992" t="s">
+      <c r="AF9" s="989"/>
+      <c r="AG9" s="990"/>
+      <c r="AH9" s="988" t="s">
         <v>59</v>
       </c>
-      <c r="AI9" s="993"/>
-      <c r="AJ9" s="994"/>
-      <c r="AK9" s="992" t="s">
+      <c r="AI9" s="989"/>
+      <c r="AJ9" s="990"/>
+      <c r="AK9" s="988" t="s">
         <v>60</v>
       </c>
-      <c r="AL9" s="993"/>
-      <c r="AM9" s="994"/>
-      <c r="AN9" s="992" t="s">
+      <c r="AL9" s="989"/>
+      <c r="AM9" s="990"/>
+      <c r="AN9" s="988" t="s">
         <v>61</v>
       </c>
-      <c r="AO9" s="993"/>
-      <c r="AP9" s="994"/>
-      <c r="AQ9" s="992" t="s">
+      <c r="AO9" s="989"/>
+      <c r="AP9" s="990"/>
+      <c r="AQ9" s="988" t="s">
         <v>62</v>
       </c>
-      <c r="AR9" s="993"/>
-      <c r="AS9" s="994"/>
-      <c r="AT9" s="992" t="s">
+      <c r="AR9" s="989"/>
+      <c r="AS9" s="990"/>
+      <c r="AT9" s="988" t="s">
         <v>63</v>
       </c>
-      <c r="AU9" s="993"/>
-      <c r="AV9" s="994"/>
+      <c r="AU9" s="989"/>
+      <c r="AV9" s="990"/>
     </row>
     <row r="10" spans="2:55" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B10" s="33" t="s">
@@ -33833,11 +33833,11 @@
       <c r="I25" s="60">
         <v>0.75</v>
       </c>
-      <c r="J25" s="977" t="s">
+      <c r="J25" s="979" t="s">
         <v>46</v>
       </c>
-      <c r="K25" s="978"/>
-      <c r="L25" s="979"/>
+      <c r="K25" s="980"/>
+      <c r="L25" s="981"/>
       <c r="Q25" s="25"/>
       <c r="R25" s="25"/>
       <c r="S25" s="25"/>
@@ -33862,16 +33862,16 @@
       <c r="I26" s="31" t="s">
         <v>12</v>
       </c>
-      <c r="J26" s="980"/>
-      <c r="K26" s="981"/>
-      <c r="L26" s="982"/>
+      <c r="J26" s="982"/>
+      <c r="K26" s="983"/>
+      <c r="L26" s="984"/>
       <c r="Q26" s="25"/>
       <c r="R26" s="25"/>
-      <c r="S26" s="986" t="s">
+      <c r="S26" s="1001" t="s">
         <v>43</v>
       </c>
-      <c r="T26" s="987"/>
-      <c r="U26" s="988"/>
+      <c r="T26" s="1002"/>
+      <c r="U26" s="1003"/>
       <c r="AI26" s="73">
         <v>1.5</v>
       </c>
@@ -33895,9 +33895,9 @@
         <f>H27*2.54*10</f>
         <v>25.4</v>
       </c>
-      <c r="J27" s="983"/>
-      <c r="K27" s="984"/>
-      <c r="L27" s="985"/>
+      <c r="J27" s="985"/>
+      <c r="K27" s="986"/>
+      <c r="L27" s="987"/>
       <c r="Q27" s="25"/>
       <c r="R27" s="25"/>
       <c r="S27" s="42"/>
@@ -34065,11 +34065,11 @@
       <c r="U32" s="54"/>
     </row>
     <row r="33" spans="3:21" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="C33" s="998"/>
-      <c r="D33" s="998"/>
-      <c r="E33" s="998"/>
-      <c r="F33" s="998"/>
-      <c r="G33" s="998"/>
+      <c r="C33" s="974"/>
+      <c r="D33" s="974"/>
+      <c r="E33" s="974"/>
+      <c r="F33" s="974"/>
+      <c r="G33" s="974"/>
       <c r="H33" s="54"/>
       <c r="I33" s="54"/>
       <c r="J33" s="54"/>
@@ -34097,20 +34097,22 @@
     <row r="35" spans="3:21" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <mergeCells count="46">
-    <mergeCell ref="C33:G33"/>
-    <mergeCell ref="B7:C8"/>
-    <mergeCell ref="D7:F9"/>
-    <mergeCell ref="J9:L9"/>
-    <mergeCell ref="J8:L8"/>
-    <mergeCell ref="H7:I7"/>
-    <mergeCell ref="H8:I8"/>
-    <mergeCell ref="AB9:AD9"/>
-    <mergeCell ref="M8:O8"/>
-    <mergeCell ref="M9:O9"/>
-    <mergeCell ref="P8:R8"/>
-    <mergeCell ref="P9:R9"/>
-    <mergeCell ref="S8:U8"/>
-    <mergeCell ref="S9:U9"/>
+    <mergeCell ref="B5:F5"/>
+    <mergeCell ref="H6:AS6"/>
+    <mergeCell ref="H5:AS5"/>
+    <mergeCell ref="J25:L27"/>
+    <mergeCell ref="S26:U26"/>
+    <mergeCell ref="S7:U7"/>
+    <mergeCell ref="Y7:AA7"/>
+    <mergeCell ref="AH7:AJ7"/>
+    <mergeCell ref="AN7:AP7"/>
+    <mergeCell ref="AQ7:AS7"/>
+    <mergeCell ref="AN9:AP9"/>
+    <mergeCell ref="AQ8:AS8"/>
+    <mergeCell ref="AQ9:AS9"/>
+    <mergeCell ref="Y8:AA8"/>
+    <mergeCell ref="Y9:AA9"/>
+    <mergeCell ref="AB8:AD8"/>
     <mergeCell ref="AT8:AV8"/>
     <mergeCell ref="AT9:AV9"/>
     <mergeCell ref="AN8:AP8"/>
@@ -34127,22 +34129,20 @@
     <mergeCell ref="AK9:AM9"/>
     <mergeCell ref="V8:X8"/>
     <mergeCell ref="V9:X9"/>
-    <mergeCell ref="B5:F5"/>
-    <mergeCell ref="H6:AS6"/>
-    <mergeCell ref="H5:AS5"/>
-    <mergeCell ref="J25:L27"/>
-    <mergeCell ref="S26:U26"/>
-    <mergeCell ref="S7:U7"/>
-    <mergeCell ref="Y7:AA7"/>
-    <mergeCell ref="AH7:AJ7"/>
-    <mergeCell ref="AN7:AP7"/>
-    <mergeCell ref="AQ7:AS7"/>
-    <mergeCell ref="AN9:AP9"/>
-    <mergeCell ref="AQ8:AS8"/>
-    <mergeCell ref="AQ9:AS9"/>
-    <mergeCell ref="Y8:AA8"/>
-    <mergeCell ref="Y9:AA9"/>
-    <mergeCell ref="AB8:AD8"/>
+    <mergeCell ref="AB9:AD9"/>
+    <mergeCell ref="M8:O8"/>
+    <mergeCell ref="M9:O9"/>
+    <mergeCell ref="P8:R8"/>
+    <mergeCell ref="P9:R9"/>
+    <mergeCell ref="S8:U8"/>
+    <mergeCell ref="S9:U9"/>
+    <mergeCell ref="C33:G33"/>
+    <mergeCell ref="B7:C8"/>
+    <mergeCell ref="D7:F9"/>
+    <mergeCell ref="J9:L9"/>
+    <mergeCell ref="J8:L8"/>
+    <mergeCell ref="H7:I7"/>
+    <mergeCell ref="H8:I8"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.78740157480314965" right="0.78740157480314965" top="0.78740157480314965" bottom="0.39370078740157483" header="0" footer="0"/>
@@ -34251,39 +34251,39 @@
       <c r="Z5" s="315"/>
     </row>
     <row r="6" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="849" t="s">
+      <c r="A6" s="833" t="s">
         <v>2</v>
       </c>
-      <c r="B6" s="849"/>
-      <c r="C6" s="849"/>
-      <c r="D6" s="849"/>
-      <c r="E6" s="849"/>
-      <c r="F6" s="849"/>
-      <c r="G6" s="849"/>
-      <c r="H6" s="849"/>
-      <c r="I6" s="849"/>
-      <c r="J6" s="849"/>
-      <c r="K6" s="849"/>
-      <c r="L6" s="849"/>
-      <c r="M6" s="849"/>
+      <c r="B6" s="833"/>
+      <c r="C6" s="833"/>
+      <c r="D6" s="833"/>
+      <c r="E6" s="833"/>
+      <c r="F6" s="833"/>
+      <c r="G6" s="833"/>
+      <c r="H6" s="833"/>
+      <c r="I6" s="833"/>
+      <c r="J6" s="833"/>
+      <c r="K6" s="833"/>
+      <c r="L6" s="833"/>
+      <c r="M6" s="833"/>
       <c r="Z6" s="315"/>
     </row>
     <row r="7" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="850">
+      <c r="A7" s="834">
         <v>1</v>
       </c>
-      <c r="B7" s="850"/>
-      <c r="C7" s="850"/>
-      <c r="D7" s="850"/>
-      <c r="E7" s="850"/>
-      <c r="F7" s="850"/>
-      <c r="G7" s="850"/>
-      <c r="H7" s="850"/>
-      <c r="I7" s="850"/>
-      <c r="J7" s="850"/>
-      <c r="K7" s="850"/>
-      <c r="L7" s="850"/>
-      <c r="M7" s="850"/>
+      <c r="B7" s="834"/>
+      <c r="C7" s="834"/>
+      <c r="D7" s="834"/>
+      <c r="E7" s="834"/>
+      <c r="F7" s="834"/>
+      <c r="G7" s="834"/>
+      <c r="H7" s="834"/>
+      <c r="I7" s="834"/>
+      <c r="J7" s="834"/>
+      <c r="K7" s="834"/>
+      <c r="L7" s="834"/>
+      <c r="M7" s="834"/>
     </row>
     <row r="8" spans="1:26" ht="8.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="9" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -34326,10 +34326,10 @@
       <c r="K10" s="285" t="s">
         <v>356</v>
       </c>
-      <c r="L10" s="851">
+      <c r="L10" s="835">
         <v>1</v>
       </c>
-      <c r="M10" s="851"/>
+      <c r="M10" s="835"/>
       <c r="N10" s="320"/>
       <c r="O10" s="320"/>
       <c r="P10" s="320"/>
@@ -34361,8 +34361,8 @@
       <c r="K11" s="285" t="s">
         <v>127</v>
       </c>
-      <c r="L11" s="847"/>
-      <c r="M11" s="847"/>
+      <c r="L11" s="836"/>
+      <c r="M11" s="836"/>
       <c r="N11" s="320"/>
       <c r="O11" s="320"/>
       <c r="P11" s="320"/>
@@ -34436,21 +34436,21 @@
       <c r="Y13" s="320"/>
     </row>
     <row r="14" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="835" t="s">
+      <c r="A14" s="846" t="s">
         <v>128</v>
       </c>
-      <c r="B14" s="836"/>
-      <c r="C14" s="836"/>
-      <c r="D14" s="836"/>
-      <c r="E14" s="836"/>
-      <c r="F14" s="836"/>
-      <c r="G14" s="836"/>
-      <c r="H14" s="836"/>
-      <c r="I14" s="836"/>
-      <c r="J14" s="836"/>
-      <c r="K14" s="836"/>
-      <c r="L14" s="836"/>
-      <c r="M14" s="837"/>
+      <c r="B14" s="847"/>
+      <c r="C14" s="847"/>
+      <c r="D14" s="847"/>
+      <c r="E14" s="847"/>
+      <c r="F14" s="847"/>
+      <c r="G14" s="847"/>
+      <c r="H14" s="847"/>
+      <c r="I14" s="847"/>
+      <c r="J14" s="847"/>
+      <c r="K14" s="847"/>
+      <c r="L14" s="847"/>
+      <c r="M14" s="848"/>
       <c r="N14" s="320"/>
       <c r="O14" s="320"/>
       <c r="P14" s="320"/>
@@ -34465,21 +34465,21 @@
       <c r="Y14" s="320"/>
     </row>
     <row r="15" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="838" t="s">
+      <c r="A15" s="849" t="s">
         <v>131</v>
       </c>
-      <c r="B15" s="839"/>
-      <c r="C15" s="839"/>
-      <c r="D15" s="839"/>
-      <c r="E15" s="839"/>
-      <c r="F15" s="839"/>
-      <c r="G15" s="839"/>
-      <c r="H15" s="839"/>
-      <c r="I15" s="839"/>
-      <c r="J15" s="839"/>
-      <c r="K15" s="839"/>
-      <c r="L15" s="839"/>
-      <c r="M15" s="840"/>
+      <c r="B15" s="850"/>
+      <c r="C15" s="850"/>
+      <c r="D15" s="850"/>
+      <c r="E15" s="850"/>
+      <c r="F15" s="850"/>
+      <c r="G15" s="850"/>
+      <c r="H15" s="850"/>
+      <c r="I15" s="850"/>
+      <c r="J15" s="850"/>
+      <c r="K15" s="850"/>
+      <c r="L15" s="850"/>
+      <c r="M15" s="851"/>
       <c r="N15" s="320"/>
       <c r="O15" s="320"/>
       <c r="P15" s="320"/>
@@ -34554,10 +34554,10 @@
       <c r="K18" s="285" t="s">
         <v>153</v>
       </c>
-      <c r="L18" s="845">
+      <c r="L18" s="856">
         <v>1</v>
       </c>
-      <c r="M18" s="846"/>
+      <c r="M18" s="857"/>
       <c r="Y18" s="320"/>
     </row>
     <row r="19" spans="1:29" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -34576,8 +34576,8 @@
       <c r="K19" s="285" t="s">
         <v>125</v>
       </c>
-      <c r="L19" s="847"/>
-      <c r="M19" s="848"/>
+      <c r="L19" s="836"/>
+      <c r="M19" s="858"/>
       <c r="Y19" s="320"/>
     </row>
     <row r="20" spans="1:29" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -34596,8 +34596,8 @@
       <c r="K20" s="285" t="s">
         <v>126</v>
       </c>
-      <c r="L20" s="847"/>
-      <c r="M20" s="848"/>
+      <c r="L20" s="836"/>
+      <c r="M20" s="858"/>
       <c r="Y20" s="320"/>
     </row>
     <row r="21" spans="1:29" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -34652,24 +34652,24 @@
       <c r="A23" s="356"/>
       <c r="B23" s="364"/>
       <c r="C23" s="364"/>
-      <c r="D23" s="841" t="s">
+      <c r="D23" s="852" t="s">
         <v>353</v>
       </c>
-      <c r="E23" s="842"/>
-      <c r="F23" s="833" t="s">
+      <c r="E23" s="853"/>
+      <c r="F23" s="843" t="s">
         <v>276</v>
       </c>
-      <c r="G23" s="833" t="s">
+      <c r="G23" s="843" t="s">
         <v>346</v>
       </c>
-      <c r="H23" s="833" t="s">
+      <c r="H23" s="843" t="s">
         <v>275</v>
       </c>
       <c r="I23" s="337"/>
-      <c r="J23" s="853" t="s">
+      <c r="J23" s="838" t="s">
         <v>146</v>
       </c>
-      <c r="K23" s="854"/>
+      <c r="K23" s="839"/>
       <c r="L23" s="497"/>
       <c r="M23" s="357"/>
       <c r="N23" s="320"/>
@@ -34684,11 +34684,11 @@
       <c r="W23" s="320"/>
       <c r="X23" s="320"/>
       <c r="Y23" s="332"/>
-      <c r="AA23" s="843" t="s">
+      <c r="AA23" s="854" t="s">
         <v>278</v>
       </c>
-      <c r="AB23" s="844"/>
-      <c r="AC23" s="833" t="s">
+      <c r="AB23" s="855"/>
+      <c r="AC23" s="843" t="s">
         <v>275</v>
       </c>
     </row>
@@ -34702,12 +34702,12 @@
       <c r="E24" s="500" t="s">
         <v>380</v>
       </c>
-      <c r="F24" s="834"/>
-      <c r="G24" s="834"/>
-      <c r="H24" s="834"/>
+      <c r="F24" s="844"/>
+      <c r="G24" s="844"/>
+      <c r="H24" s="844"/>
       <c r="I24" s="337"/>
-      <c r="J24" s="855"/>
-      <c r="K24" s="856"/>
+      <c r="J24" s="840"/>
+      <c r="K24" s="841"/>
       <c r="L24" s="497"/>
       <c r="M24" s="358"/>
       <c r="N24" s="320"/>
@@ -34728,7 +34728,7 @@
       <c r="AB24" s="380" t="s">
         <v>12</v>
       </c>
-      <c r="AC24" s="834"/>
+      <c r="AC24" s="844"/>
     </row>
     <row r="25" spans="1:29" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="356"/>
@@ -35136,7 +35136,7 @@
       <c r="J32" s="298"/>
       <c r="K32" s="298"/>
       <c r="L32" s="298"/>
-      <c r="M32" s="858"/>
+      <c r="M32" s="845"/>
       <c r="N32" s="320"/>
       <c r="O32" s="320"/>
       <c r="P32" s="320"/>
@@ -35186,7 +35186,7 @@
       <c r="J33" s="298"/>
       <c r="K33" s="298"/>
       <c r="L33" s="298"/>
-      <c r="M33" s="858"/>
+      <c r="M33" s="845"/>
       <c r="N33" s="320"/>
       <c r="O33" s="320"/>
       <c r="P33" s="320"/>
@@ -36048,21 +36048,21 @@
       <c r="Z59" s="480"/>
     </row>
     <row r="60" spans="1:26" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A60" s="857" t="s">
+      <c r="A60" s="842" t="s">
         <v>296</v>
       </c>
-      <c r="B60" s="857"/>
-      <c r="C60" s="857"/>
-      <c r="D60" s="857"/>
-      <c r="E60" s="857"/>
-      <c r="F60" s="857"/>
-      <c r="G60" s="857"/>
-      <c r="H60" s="857"/>
-      <c r="I60" s="857"/>
-      <c r="J60" s="857"/>
-      <c r="K60" s="857"/>
-      <c r="L60" s="857"/>
-      <c r="M60" s="857"/>
+      <c r="B60" s="842"/>
+      <c r="C60" s="842"/>
+      <c r="D60" s="842"/>
+      <c r="E60" s="842"/>
+      <c r="F60" s="842"/>
+      <c r="G60" s="842"/>
+      <c r="H60" s="842"/>
+      <c r="I60" s="842"/>
+      <c r="J60" s="842"/>
+      <c r="K60" s="842"/>
+      <c r="L60" s="842"/>
+      <c r="M60" s="842"/>
       <c r="N60" s="483"/>
       <c r="O60" s="483"/>
       <c r="P60" s="483"/>
@@ -36108,21 +36108,21 @@
       <c r="Z61" s="480"/>
     </row>
     <row r="62" spans="1:26" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A62" s="857" t="s">
+      <c r="A62" s="842" t="s">
         <v>355</v>
       </c>
-      <c r="B62" s="857"/>
-      <c r="C62" s="857"/>
-      <c r="D62" s="857"/>
-      <c r="E62" s="857"/>
-      <c r="F62" s="857"/>
-      <c r="G62" s="857"/>
-      <c r="H62" s="857"/>
-      <c r="I62" s="857"/>
-      <c r="J62" s="857"/>
-      <c r="K62" s="857"/>
-      <c r="L62" s="857"/>
-      <c r="M62" s="857"/>
+      <c r="B62" s="842"/>
+      <c r="C62" s="842"/>
+      <c r="D62" s="842"/>
+      <c r="E62" s="842"/>
+      <c r="F62" s="842"/>
+      <c r="G62" s="842"/>
+      <c r="H62" s="842"/>
+      <c r="I62" s="842"/>
+      <c r="J62" s="842"/>
+      <c r="K62" s="842"/>
+      <c r="L62" s="842"/>
+      <c r="M62" s="842"/>
       <c r="N62" s="319"/>
       <c r="O62" s="319"/>
       <c r="P62" s="319"/>
@@ -36193,12 +36193,12 @@
       <c r="Z64" s="482"/>
     </row>
     <row r="65" spans="1:13" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A65" s="852" t="s">
+      <c r="A65" s="837" t="s">
         <v>362</v>
       </c>
-      <c r="B65" s="852"/>
-      <c r="C65" s="852"/>
-      <c r="D65" s="852"/>
+      <c r="B65" s="837"/>
+      <c r="C65" s="837"/>
+      <c r="D65" s="837"/>
       <c r="E65" s="337"/>
       <c r="F65" s="337"/>
       <c r="G65" s="337"/>
@@ -36280,6 +36280,15 @@
     <protectedRange sqref="D9:D10" name="Rango3_3_1_1_1_1_1_2_1_1_1"/>
   </protectedRanges>
   <mergeCells count="20">
+    <mergeCell ref="AC23:AC24"/>
+    <mergeCell ref="A14:M14"/>
+    <mergeCell ref="A15:M15"/>
+    <mergeCell ref="D23:E23"/>
+    <mergeCell ref="F23:F24"/>
+    <mergeCell ref="AA23:AB23"/>
+    <mergeCell ref="L18:M18"/>
+    <mergeCell ref="L19:M19"/>
+    <mergeCell ref="L20:M20"/>
     <mergeCell ref="A6:M6"/>
     <mergeCell ref="A7:M7"/>
     <mergeCell ref="L10:M10"/>
@@ -36291,15 +36300,6 @@
     <mergeCell ref="H23:H24"/>
     <mergeCell ref="A62:M62"/>
     <mergeCell ref="M32:M33"/>
-    <mergeCell ref="AC23:AC24"/>
-    <mergeCell ref="A14:M14"/>
-    <mergeCell ref="A15:M15"/>
-    <mergeCell ref="D23:E23"/>
-    <mergeCell ref="F23:F24"/>
-    <mergeCell ref="AA23:AB23"/>
-    <mergeCell ref="L18:M18"/>
-    <mergeCell ref="L19:M19"/>
-    <mergeCell ref="L20:M20"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0" right="0" top="0.59055118110236227" bottom="0" header="0.11811023622047245" footer="0"/>
@@ -36407,37 +36407,37 @@
       <c r="Y5" s="315"/>
     </row>
     <row r="6" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="849" t="s">
+      <c r="A6" s="833" t="s">
         <v>2</v>
       </c>
-      <c r="B6" s="849"/>
-      <c r="C6" s="849"/>
-      <c r="D6" s="849"/>
-      <c r="E6" s="849"/>
-      <c r="F6" s="849"/>
-      <c r="G6" s="849"/>
-      <c r="H6" s="849"/>
-      <c r="I6" s="849"/>
-      <c r="J6" s="849"/>
-      <c r="K6" s="849"/>
-      <c r="L6" s="849"/>
+      <c r="B6" s="833"/>
+      <c r="C6" s="833"/>
+      <c r="D6" s="833"/>
+      <c r="E6" s="833"/>
+      <c r="F6" s="833"/>
+      <c r="G6" s="833"/>
+      <c r="H6" s="833"/>
+      <c r="I6" s="833"/>
+      <c r="J6" s="833"/>
+      <c r="K6" s="833"/>
+      <c r="L6" s="833"/>
       <c r="Y6" s="315"/>
     </row>
     <row r="7" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="867">
+      <c r="A7" s="859">
         <v>1</v>
       </c>
-      <c r="B7" s="867"/>
-      <c r="C7" s="867"/>
-      <c r="D7" s="867"/>
-      <c r="E7" s="867"/>
-      <c r="F7" s="867"/>
-      <c r="G7" s="867"/>
-      <c r="H7" s="867"/>
-      <c r="I7" s="867"/>
-      <c r="J7" s="867"/>
-      <c r="K7" s="867"/>
-      <c r="L7" s="867"/>
+      <c r="B7" s="859"/>
+      <c r="C7" s="859"/>
+      <c r="D7" s="859"/>
+      <c r="E7" s="859"/>
+      <c r="F7" s="859"/>
+      <c r="G7" s="859"/>
+      <c r="H7" s="859"/>
+      <c r="I7" s="859"/>
+      <c r="J7" s="859"/>
+      <c r="K7" s="859"/>
+      <c r="L7" s="859"/>
     </row>
     <row r="8" spans="1:25" ht="8.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="9" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -36608,20 +36608,20 @@
       <c r="X13" s="320"/>
     </row>
     <row r="14" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="835" t="s">
+      <c r="A14" s="846" t="s">
         <v>128</v>
       </c>
-      <c r="B14" s="836"/>
-      <c r="C14" s="836"/>
-      <c r="D14" s="836"/>
-      <c r="E14" s="836"/>
-      <c r="F14" s="836"/>
-      <c r="G14" s="836"/>
-      <c r="H14" s="836"/>
-      <c r="I14" s="836"/>
-      <c r="J14" s="836"/>
-      <c r="K14" s="836"/>
-      <c r="L14" s="837"/>
+      <c r="B14" s="847"/>
+      <c r="C14" s="847"/>
+      <c r="D14" s="847"/>
+      <c r="E14" s="847"/>
+      <c r="F14" s="847"/>
+      <c r="G14" s="847"/>
+      <c r="H14" s="847"/>
+      <c r="I14" s="847"/>
+      <c r="J14" s="847"/>
+      <c r="K14" s="847"/>
+      <c r="L14" s="848"/>
       <c r="M14" s="320"/>
       <c r="N14" s="320"/>
       <c r="O14" s="320"/>
@@ -36636,20 +36636,20 @@
       <c r="X14" s="320"/>
     </row>
     <row r="15" spans="1:25" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="838" t="s">
+      <c r="A15" s="849" t="s">
         <v>466</v>
       </c>
-      <c r="B15" s="839"/>
-      <c r="C15" s="839"/>
-      <c r="D15" s="839"/>
-      <c r="E15" s="839"/>
-      <c r="F15" s="839"/>
-      <c r="G15" s="839"/>
-      <c r="H15" s="839"/>
-      <c r="I15" s="839"/>
-      <c r="J15" s="839"/>
-      <c r="K15" s="839"/>
-      <c r="L15" s="840"/>
+      <c r="B15" s="850"/>
+      <c r="C15" s="850"/>
+      <c r="D15" s="850"/>
+      <c r="E15" s="850"/>
+      <c r="F15" s="850"/>
+      <c r="G15" s="850"/>
+      <c r="H15" s="850"/>
+      <c r="I15" s="850"/>
+      <c r="J15" s="850"/>
+      <c r="K15" s="850"/>
+      <c r="L15" s="851"/>
       <c r="M15" s="320"/>
       <c r="N15" s="320"/>
       <c r="O15" s="320"/>
@@ -36835,30 +36835,30 @@
       <c r="A23" s="356"/>
       <c r="B23" s="364"/>
       <c r="C23" s="364"/>
-      <c r="D23" s="841" t="s">
+      <c r="D23" s="852" t="s">
         <v>353</v>
       </c>
-      <c r="E23" s="842"/>
-      <c r="F23" s="833" t="s">
+      <c r="E23" s="853"/>
+      <c r="F23" s="843" t="s">
         <v>276</v>
       </c>
-      <c r="G23" s="833" t="s">
+      <c r="G23" s="843" t="s">
         <v>346</v>
       </c>
-      <c r="H23" s="833" t="s">
+      <c r="H23" s="843" t="s">
         <v>275</v>
       </c>
       <c r="I23" s="337"/>
-      <c r="J23" s="853" t="s">
+      <c r="J23" s="838" t="s">
         <v>146</v>
       </c>
-      <c r="K23" s="854"/>
+      <c r="K23" s="839"/>
       <c r="L23" s="651"/>
       <c r="M23" s="320"/>
-      <c r="N23" s="853" t="s">
+      <c r="N23" s="838" t="s">
         <v>146</v>
       </c>
-      <c r="O23" s="854"/>
+      <c r="O23" s="839"/>
       <c r="P23" s="320"/>
       <c r="Q23" s="320"/>
       <c r="R23" s="320"/>
@@ -36868,11 +36868,11 @@
       <c r="V23" s="320"/>
       <c r="W23" s="320"/>
       <c r="X23" s="332"/>
-      <c r="Z23" s="843" t="s">
+      <c r="Z23" s="854" t="s">
         <v>278</v>
       </c>
-      <c r="AA23" s="844"/>
-      <c r="AB23" s="833" t="s">
+      <c r="AA23" s="855"/>
+      <c r="AB23" s="843" t="s">
         <v>275</v>
       </c>
     </row>
@@ -36886,16 +36886,16 @@
       <c r="E24" s="500" t="s">
         <v>380</v>
       </c>
-      <c r="F24" s="834"/>
-      <c r="G24" s="834"/>
-      <c r="H24" s="834"/>
+      <c r="F24" s="844"/>
+      <c r="G24" s="844"/>
+      <c r="H24" s="844"/>
       <c r="I24" s="337"/>
-      <c r="J24" s="855"/>
-      <c r="K24" s="856"/>
+      <c r="J24" s="840"/>
+      <c r="K24" s="841"/>
       <c r="L24" s="651"/>
       <c r="M24" s="320"/>
-      <c r="N24" s="855"/>
-      <c r="O24" s="856"/>
+      <c r="N24" s="840"/>
+      <c r="O24" s="841"/>
       <c r="P24" s="320"/>
       <c r="Q24" s="320"/>
       <c r="R24" s="320"/>
@@ -36911,7 +36911,7 @@
       <c r="AA24" s="380" t="s">
         <v>12</v>
       </c>
-      <c r="AB24" s="834"/>
+      <c r="AB24" s="844"/>
     </row>
     <row r="25" spans="1:28" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="356"/>
@@ -36936,10 +36936,10 @@
         <v>#DIV/0!</v>
       </c>
       <c r="I25" s="337"/>
-      <c r="J25" s="860" t="s">
+      <c r="J25" s="861" t="s">
         <v>381</v>
       </c>
-      <c r="K25" s="863" t="e">
+      <c r="K25" s="864" t="e">
         <f>+datos!I21</f>
         <v>#DIV/0!</v>
       </c>
@@ -36995,8 +36995,8 @@
         <v>#DIV/0!</v>
       </c>
       <c r="I26" s="337"/>
-      <c r="J26" s="861"/>
-      <c r="K26" s="864"/>
+      <c r="J26" s="862"/>
+      <c r="K26" s="865"/>
       <c r="L26" s="652"/>
       <c r="M26" s="320"/>
       <c r="N26" s="360" t="s">
@@ -37049,8 +37049,8 @@
         <v>#DIV/0!</v>
       </c>
       <c r="I27" s="337"/>
-      <c r="J27" s="862"/>
-      <c r="K27" s="865"/>
+      <c r="J27" s="863"/>
+      <c r="K27" s="866"/>
       <c r="L27" s="648"/>
       <c r="M27" s="320"/>
       <c r="N27" s="360" t="s">
@@ -38150,37 +38150,37 @@
       <c r="Y57" s="386"/>
     </row>
     <row r="58" spans="1:25" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A58" s="866" t="s">
+      <c r="A58" s="867" t="s">
         <v>467</v>
       </c>
-      <c r="B58" s="866"/>
-      <c r="C58" s="866"/>
-      <c r="D58" s="866"/>
-      <c r="E58" s="866"/>
-      <c r="F58" s="866"/>
-      <c r="G58" s="866"/>
-      <c r="H58" s="866"/>
-      <c r="I58" s="866"/>
-      <c r="J58" s="866"/>
-      <c r="K58" s="866"/>
-      <c r="L58" s="866"/>
+      <c r="B58" s="867"/>
+      <c r="C58" s="867"/>
+      <c r="D58" s="867"/>
+      <c r="E58" s="867"/>
+      <c r="F58" s="867"/>
+      <c r="G58" s="867"/>
+      <c r="H58" s="867"/>
+      <c r="I58" s="867"/>
+      <c r="J58" s="867"/>
+      <c r="K58" s="867"/>
+      <c r="L58" s="867"/>
       <c r="Y58" s="386"/>
     </row>
     <row r="59" spans="1:25" ht="26.4" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A59" s="859" t="s">
+      <c r="A59" s="860" t="s">
         <v>468</v>
       </c>
-      <c r="B59" s="859"/>
-      <c r="C59" s="859"/>
-      <c r="D59" s="859"/>
-      <c r="E59" s="859"/>
-      <c r="F59" s="859"/>
-      <c r="G59" s="859"/>
-      <c r="H59" s="859"/>
-      <c r="I59" s="859"/>
-      <c r="J59" s="859"/>
-      <c r="K59" s="859"/>
-      <c r="L59" s="859"/>
+      <c r="B59" s="860"/>
+      <c r="C59" s="860"/>
+      <c r="D59" s="860"/>
+      <c r="E59" s="860"/>
+      <c r="F59" s="860"/>
+      <c r="G59" s="860"/>
+      <c r="H59" s="860"/>
+      <c r="I59" s="860"/>
+      <c r="J59" s="860"/>
+      <c r="K59" s="860"/>
+      <c r="L59" s="860"/>
       <c r="M59" s="319"/>
       <c r="N59" s="319"/>
       <c r="O59" s="319"/>
@@ -38196,20 +38196,20 @@
       <c r="Y59" s="480"/>
     </row>
     <row r="60" spans="1:25" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A60" s="859" t="s">
+      <c r="A60" s="860" t="s">
         <v>469</v>
       </c>
-      <c r="B60" s="859"/>
-      <c r="C60" s="859"/>
-      <c r="D60" s="859"/>
-      <c r="E60" s="859"/>
-      <c r="F60" s="859"/>
-      <c r="G60" s="859"/>
-      <c r="H60" s="859"/>
-      <c r="I60" s="859"/>
-      <c r="J60" s="859"/>
-      <c r="K60" s="859"/>
-      <c r="L60" s="859"/>
+      <c r="B60" s="860"/>
+      <c r="C60" s="860"/>
+      <c r="D60" s="860"/>
+      <c r="E60" s="860"/>
+      <c r="F60" s="860"/>
+      <c r="G60" s="860"/>
+      <c r="H60" s="860"/>
+      <c r="I60" s="860"/>
+      <c r="J60" s="860"/>
+      <c r="K60" s="860"/>
+      <c r="L60" s="860"/>
       <c r="M60" s="483"/>
       <c r="N60" s="483"/>
       <c r="O60" s="483"/>
@@ -38225,20 +38225,20 @@
       <c r="Y60" s="483"/>
     </row>
     <row r="61" spans="1:25" ht="22.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A61" s="859" t="s">
+      <c r="A61" s="860" t="s">
         <v>470</v>
       </c>
-      <c r="B61" s="859"/>
-      <c r="C61" s="859"/>
-      <c r="D61" s="859"/>
-      <c r="E61" s="859"/>
-      <c r="F61" s="859"/>
-      <c r="G61" s="859"/>
-      <c r="H61" s="859"/>
-      <c r="I61" s="859"/>
-      <c r="J61" s="859"/>
-      <c r="K61" s="859"/>
-      <c r="L61" s="859"/>
+      <c r="B61" s="860"/>
+      <c r="C61" s="860"/>
+      <c r="D61" s="860"/>
+      <c r="E61" s="860"/>
+      <c r="F61" s="860"/>
+      <c r="G61" s="860"/>
+      <c r="H61" s="860"/>
+      <c r="I61" s="860"/>
+      <c r="J61" s="860"/>
+      <c r="K61" s="860"/>
+      <c r="L61" s="860"/>
       <c r="M61" s="319"/>
       <c r="N61" s="319"/>
       <c r="O61" s="319"/>
@@ -38254,20 +38254,20 @@
       <c r="Y61" s="480"/>
     </row>
     <row r="62" spans="1:25" ht="26.4" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A62" s="857" t="s">
+      <c r="A62" s="842" t="s">
         <v>471</v>
       </c>
-      <c r="B62" s="857"/>
-      <c r="C62" s="857"/>
-      <c r="D62" s="857"/>
-      <c r="E62" s="857"/>
-      <c r="F62" s="857"/>
-      <c r="G62" s="857"/>
-      <c r="H62" s="857"/>
-      <c r="I62" s="857"/>
-      <c r="J62" s="857"/>
-      <c r="K62" s="857"/>
-      <c r="L62" s="857"/>
+      <c r="B62" s="842"/>
+      <c r="C62" s="842"/>
+      <c r="D62" s="842"/>
+      <c r="E62" s="842"/>
+      <c r="F62" s="842"/>
+      <c r="G62" s="842"/>
+      <c r="H62" s="842"/>
+      <c r="I62" s="842"/>
+      <c r="J62" s="842"/>
+      <c r="K62" s="842"/>
+      <c r="L62" s="842"/>
       <c r="M62" s="319"/>
       <c r="N62" s="319"/>
       <c r="O62" s="319"/>
@@ -38337,12 +38337,12 @@
       <c r="Y64" s="482"/>
     </row>
     <row r="65" spans="1:12" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A65" s="852" t="s">
+      <c r="A65" s="837" t="s">
         <v>472</v>
       </c>
-      <c r="B65" s="852"/>
-      <c r="C65" s="852"/>
-      <c r="D65" s="852"/>
+      <c r="B65" s="837"/>
+      <c r="C65" s="837"/>
+      <c r="D65" s="837"/>
       <c r="E65" s="337"/>
       <c r="F65" s="337"/>
       <c r="G65" s="337"/>
@@ -38420,11 +38420,6 @@
   </protectedRanges>
   <dataConsolidate/>
   <mergeCells count="20">
-    <mergeCell ref="A6:L6"/>
-    <mergeCell ref="A7:L7"/>
-    <mergeCell ref="A14:L14"/>
-    <mergeCell ref="A15:L15"/>
-    <mergeCell ref="Z23:AA23"/>
     <mergeCell ref="AB23:AB24"/>
     <mergeCell ref="A60:L60"/>
     <mergeCell ref="A62:L62"/>
@@ -38440,6 +38435,11 @@
     <mergeCell ref="A61:L61"/>
     <mergeCell ref="A59:L59"/>
     <mergeCell ref="A58:L58"/>
+    <mergeCell ref="A6:L6"/>
+    <mergeCell ref="A7:L7"/>
+    <mergeCell ref="A14:L14"/>
+    <mergeCell ref="A15:L15"/>
+    <mergeCell ref="Z23:AA23"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0" right="0" top="0.59055118110236227" bottom="0" header="0" footer="0"/>
@@ -38469,35 +38469,35 @@
   <sheetData>
     <row r="1" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="470"/>
-      <c r="B1" s="835" t="s">
+      <c r="B1" s="846" t="s">
         <v>128</v>
       </c>
-      <c r="C1" s="836"/>
-      <c r="D1" s="836"/>
-      <c r="E1" s="836"/>
-      <c r="F1" s="836"/>
-      <c r="G1" s="836"/>
-      <c r="H1" s="836"/>
-      <c r="I1" s="836"/>
-      <c r="J1" s="836"/>
-      <c r="K1" s="836"/>
-      <c r="L1" s="837"/>
+      <c r="C1" s="847"/>
+      <c r="D1" s="847"/>
+      <c r="E1" s="847"/>
+      <c r="F1" s="847"/>
+      <c r="G1" s="847"/>
+      <c r="H1" s="847"/>
+      <c r="I1" s="847"/>
+      <c r="J1" s="847"/>
+      <c r="K1" s="847"/>
+      <c r="L1" s="848"/>
     </row>
     <row r="2" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="470"/>
-      <c r="B2" s="838" t="s">
+      <c r="B2" s="849" t="s">
         <v>383</v>
       </c>
-      <c r="C2" s="839"/>
-      <c r="D2" s="839"/>
-      <c r="E2" s="839"/>
-      <c r="F2" s="839"/>
-      <c r="G2" s="839"/>
-      <c r="H2" s="839"/>
-      <c r="I2" s="839"/>
-      <c r="J2" s="839"/>
-      <c r="K2" s="839"/>
-      <c r="L2" s="840"/>
+      <c r="C2" s="850"/>
+      <c r="D2" s="850"/>
+      <c r="E2" s="850"/>
+      <c r="F2" s="850"/>
+      <c r="G2" s="850"/>
+      <c r="H2" s="850"/>
+      <c r="I2" s="850"/>
+      <c r="J2" s="850"/>
+      <c r="K2" s="850"/>
+      <c r="L2" s="851"/>
     </row>
     <row r="3" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="470"/>
@@ -38765,7 +38765,7 @@
         <v>285</v>
       </c>
       <c r="H15" s="538">
-        <f>+IF(C11="Global",FORMATO!D22,FORMATO!D36)</f>
+        <f>+IF(C10="Global",FORMATO!D22,FORMATO!D36)</f>
         <v>0</v>
       </c>
       <c r="I15" s="444">
@@ -40333,7 +40333,7 @@
     <row r="88" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="89" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="TNSh9Anr1QAwo+Wu7s6k6M95M9SOg/Gy/xVzI3YskQB47xYzcUrVU9oMmMALZnEQFevVwRVapT4xI+pocclfog==" saltValue="QcweydN+0uFY4Pu1YTEyCA==" spinCount="100000" sheet="1" selectLockedCells="1" selectUnlockedCells="1"/>
+  <sheetProtection algorithmName="SHA-512" hashValue="PhSjsJrvoH6nY17GGGXQbM6919a0pS0xFYS8BjkTuVmW528wUwejdzF3ex+AFMUD6QoE8jLqA43PhA/Jz5a1lw==" saltValue="q1DYuEWj9QoKvOAlnxc1DA==" spinCount="100000" sheet="1" selectLockedCells="1" selectUnlockedCells="1"/>
   <mergeCells count="15">
     <mergeCell ref="C47:E47"/>
     <mergeCell ref="C61:D61"/>
@@ -47945,35 +47945,35 @@
       <c r="K4" s="87"/>
     </row>
     <row r="5" spans="1:31" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="920" t="s">
+      <c r="A5" s="932" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="920"/>
-      <c r="C5" s="920"/>
-      <c r="D5" s="920"/>
-      <c r="E5" s="920"/>
-      <c r="F5" s="920"/>
-      <c r="G5" s="920"/>
-      <c r="H5" s="920"/>
-      <c r="I5" s="920"/>
-      <c r="J5" s="920"/>
-      <c r="K5" s="920"/>
+      <c r="B5" s="932"/>
+      <c r="C5" s="932"/>
+      <c r="D5" s="932"/>
+      <c r="E5" s="932"/>
+      <c r="F5" s="932"/>
+      <c r="G5" s="932"/>
+      <c r="H5" s="932"/>
+      <c r="I5" s="932"/>
+      <c r="J5" s="932"/>
+      <c r="K5" s="932"/>
     </row>
     <row r="6" spans="1:31" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="927">
+      <c r="A6" s="939">
         <f>+K12</f>
         <v>32</v>
       </c>
-      <c r="B6" s="927"/>
-      <c r="C6" s="927"/>
-      <c r="D6" s="927"/>
-      <c r="E6" s="927"/>
-      <c r="F6" s="927"/>
-      <c r="G6" s="927"/>
-      <c r="H6" s="927"/>
-      <c r="I6" s="927"/>
-      <c r="J6" s="927"/>
-      <c r="K6" s="927"/>
+      <c r="B6" s="939"/>
+      <c r="C6" s="939"/>
+      <c r="D6" s="939"/>
+      <c r="E6" s="939"/>
+      <c r="F6" s="939"/>
+      <c r="G6" s="939"/>
+      <c r="H6" s="939"/>
+      <c r="I6" s="939"/>
+      <c r="J6" s="939"/>
+      <c r="K6" s="939"/>
       <c r="S6" s="259" t="s">
         <v>101</v>
       </c>
@@ -48050,10 +48050,10 @@
       <c r="S9" s="275" t="s">
         <v>105</v>
       </c>
-      <c r="T9" s="931">
+      <c r="T9" s="943">
         <v>44090</v>
       </c>
-      <c r="U9" s="931"/>
+      <c r="U9" s="943"/>
       <c r="V9" s="276"/>
       <c r="W9" s="277"/>
       <c r="X9" s="276"/>
@@ -48198,19 +48198,19 @@
       <c r="S13" s="86"/>
     </row>
     <row r="14" spans="1:31" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="928" t="s">
+      <c r="A14" s="940" t="s">
         <v>128</v>
       </c>
-      <c r="B14" s="929"/>
-      <c r="C14" s="929"/>
-      <c r="D14" s="929"/>
-      <c r="E14" s="929"/>
-      <c r="F14" s="929"/>
-      <c r="G14" s="929"/>
-      <c r="H14" s="929"/>
-      <c r="I14" s="929"/>
-      <c r="J14" s="929"/>
-      <c r="K14" s="930"/>
+      <c r="B14" s="941"/>
+      <c r="C14" s="941"/>
+      <c r="D14" s="941"/>
+      <c r="E14" s="941"/>
+      <c r="F14" s="941"/>
+      <c r="G14" s="941"/>
+      <c r="H14" s="941"/>
+      <c r="I14" s="941"/>
+      <c r="J14" s="941"/>
+      <c r="K14" s="942"/>
       <c r="L14" s="87"/>
       <c r="M14" s="87"/>
       <c r="P14" s="86"/>
@@ -48219,19 +48219,19 @@
       <c r="S14" s="86"/>
     </row>
     <row r="15" spans="1:31" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="935" t="s">
+      <c r="A15" s="947" t="s">
         <v>131</v>
       </c>
-      <c r="B15" s="936"/>
-      <c r="C15" s="936"/>
-      <c r="D15" s="936"/>
-      <c r="E15" s="936"/>
-      <c r="F15" s="936"/>
-      <c r="G15" s="936"/>
-      <c r="H15" s="936"/>
-      <c r="I15" s="936"/>
-      <c r="J15" s="936"/>
-      <c r="K15" s="937"/>
+      <c r="B15" s="948"/>
+      <c r="C15" s="948"/>
+      <c r="D15" s="948"/>
+      <c r="E15" s="948"/>
+      <c r="F15" s="948"/>
+      <c r="G15" s="948"/>
+      <c r="H15" s="948"/>
+      <c r="I15" s="948"/>
+      <c r="J15" s="948"/>
+      <c r="K15" s="949"/>
       <c r="L15" s="87"/>
       <c r="M15" s="87"/>
       <c r="P15" s="86"/>
@@ -48259,17 +48259,17 @@
       <c r="S16" s="86"/>
     </row>
     <row r="17" spans="1:27" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="925" t="s">
+      <c r="A17" s="937" t="s">
         <v>5</v>
       </c>
-      <c r="B17" s="926"/>
-      <c r="C17" s="926"/>
-      <c r="D17" s="926"/>
-      <c r="E17" s="926"/>
-      <c r="F17" s="926"/>
-      <c r="G17" s="926"/>
-      <c r="H17" s="926"/>
-      <c r="I17" s="926"/>
+      <c r="B17" s="938"/>
+      <c r="C17" s="938"/>
+      <c r="D17" s="938"/>
+      <c r="E17" s="938"/>
+      <c r="F17" s="938"/>
+      <c r="G17" s="938"/>
+      <c r="H17" s="938"/>
+      <c r="I17" s="938"/>
       <c r="J17" s="1"/>
       <c r="K17" s="199"/>
       <c r="L17" s="87"/>
@@ -48337,23 +48337,23 @@
       <c r="Q19" s="86"/>
       <c r="R19" s="86"/>
       <c r="S19" s="86"/>
-      <c r="U19" s="939" t="s">
+      <c r="U19" s="920" t="s">
         <v>9</v>
       </c>
-      <c r="V19" s="940"/>
-      <c r="W19" s="919" t="s">
+      <c r="V19" s="921"/>
+      <c r="W19" s="931" t="s">
         <v>100</v>
       </c>
-      <c r="X19" s="833" t="s">
+      <c r="X19" s="843" t="s">
         <v>45</v>
       </c>
-      <c r="Y19" s="833" t="s">
+      <c r="Y19" s="843" t="s">
         <v>41</v>
       </c>
-      <c r="Z19" s="833" t="s">
+      <c r="Z19" s="843" t="s">
         <v>42</v>
       </c>
-      <c r="AA19" s="833" t="s">
+      <c r="AA19" s="843" t="s">
         <v>43</v>
       </c>
     </row>
@@ -48391,11 +48391,11 @@
       <c r="V20" s="187" t="s">
         <v>12</v>
       </c>
-      <c r="W20" s="919"/>
-      <c r="X20" s="834"/>
-      <c r="Y20" s="834"/>
-      <c r="Z20" s="834"/>
-      <c r="AA20" s="834"/>
+      <c r="W20" s="931"/>
+      <c r="X20" s="844"/>
+      <c r="Y20" s="844"/>
+      <c r="Z20" s="844"/>
+      <c r="AA20" s="844"/>
     </row>
     <row r="21" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="288" t="s">
@@ -48488,27 +48488,27 @@
     </row>
     <row r="23" spans="1:27" s="4" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="140"/>
-      <c r="B23" s="939" t="s">
+      <c r="B23" s="920" t="s">
         <v>9</v>
       </c>
-      <c r="C23" s="940"/>
-      <c r="D23" s="833" t="s">
+      <c r="C23" s="921"/>
+      <c r="D23" s="843" t="s">
         <v>45</v>
       </c>
-      <c r="E23" s="833" t="s">
+      <c r="E23" s="843" t="s">
         <v>41</v>
       </c>
-      <c r="F23" s="833" t="s">
+      <c r="F23" s="843" t="s">
         <v>42</v>
       </c>
-      <c r="G23" s="833" t="s">
+      <c r="G23" s="843" t="s">
         <v>43</v>
       </c>
       <c r="H23" s="138"/>
-      <c r="I23" s="944" t="s">
+      <c r="I23" s="925" t="s">
         <v>36</v>
       </c>
-      <c r="J23" s="945"/>
+      <c r="J23" s="926"/>
       <c r="K23" s="139"/>
       <c r="L23" s="91"/>
       <c r="M23" s="91"/>
@@ -48549,16 +48549,16 @@
       <c r="C24" s="187" t="s">
         <v>12</v>
       </c>
-      <c r="D24" s="834"/>
-      <c r="E24" s="834"/>
-      <c r="F24" s="834"/>
-      <c r="G24" s="834"/>
+      <c r="D24" s="844"/>
+      <c r="E24" s="844"/>
+      <c r="F24" s="844"/>
+      <c r="G24" s="844"/>
       <c r="H24" s="156"/>
-      <c r="I24" s="947">
+      <c r="I24" s="928">
         <f>+Q23</f>
         <v>23983.979695431473</v>
       </c>
-      <c r="J24" s="948"/>
+      <c r="J24" s="929"/>
       <c r="K24" s="139"/>
       <c r="L24" s="91"/>
       <c r="M24" s="91"/>
@@ -48672,10 +48672,10 @@
       </c>
       <c r="G26" s="97"/>
       <c r="H26" s="142"/>
-      <c r="I26" s="946" t="s">
+      <c r="I26" s="927" t="s">
         <v>92</v>
       </c>
-      <c r="J26" s="946"/>
+      <c r="J26" s="927"/>
       <c r="K26" s="143"/>
       <c r="L26" s="91"/>
       <c r="M26" s="91"/>
@@ -48926,16 +48926,16 @@
         <v>57.746817294661284</v>
       </c>
       <c r="H30" s="142"/>
-      <c r="I30" s="924"/>
-      <c r="J30" s="924"/>
+      <c r="I30" s="936"/>
+      <c r="J30" s="936"/>
       <c r="K30" s="143"/>
       <c r="L30" s="91"/>
-      <c r="M30" s="932" t="s">
+      <c r="M30" s="944" t="s">
         <v>74</v>
       </c>
-      <c r="N30" s="933"/>
-      <c r="O30" s="933"/>
-      <c r="P30" s="934"/>
+      <c r="N30" s="945"/>
+      <c r="O30" s="945"/>
+      <c r="P30" s="946"/>
       <c r="T30" s="99"/>
       <c r="U30" s="93" t="s">
         <v>88</v>
@@ -48988,16 +48988,16 @@
         <v>38.462771103509866</v>
       </c>
       <c r="H31" s="142"/>
-      <c r="I31" s="924"/>
-      <c r="J31" s="924"/>
+      <c r="I31" s="936"/>
+      <c r="J31" s="936"/>
       <c r="K31" s="143"/>
       <c r="L31" s="91"/>
-      <c r="M31" s="921" t="s">
+      <c r="M31" s="933" t="s">
         <v>82</v>
       </c>
-      <c r="N31" s="922"/>
-      <c r="O31" s="922"/>
-      <c r="P31" s="923"/>
+      <c r="N31" s="934"/>
+      <c r="O31" s="934"/>
+      <c r="P31" s="935"/>
       <c r="T31" s="99"/>
       <c r="U31" s="147" t="s">
         <v>90</v>
@@ -49162,11 +49162,11 @@
         <f t="shared" ref="U34:U42" si="10">+T34</f>
         <v>25.4</v>
       </c>
-      <c r="Z34" s="941" t="s">
+      <c r="Z34" s="922" t="s">
         <v>89</v>
       </c>
-      <c r="AA34" s="942"/>
-      <c r="AB34" s="942"/>
+      <c r="AA34" s="923"/>
+      <c r="AB34" s="923"/>
     </row>
     <row r="35" spans="1:28" s="4" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="140"/>
@@ -49730,14 +49730,14 @@
       </c>
       <c r="B57" s="5"/>
       <c r="C57" s="5"/>
-      <c r="D57" s="943"/>
-      <c r="E57" s="943"/>
-      <c r="F57" s="943"/>
-      <c r="G57" s="943"/>
-      <c r="H57" s="943"/>
-      <c r="I57" s="943"/>
-      <c r="J57" s="943"/>
-      <c r="K57" s="943"/>
+      <c r="D57" s="924"/>
+      <c r="E57" s="924"/>
+      <c r="F57" s="924"/>
+      <c r="G57" s="924"/>
+      <c r="H57" s="924"/>
+      <c r="I57" s="924"/>
+      <c r="J57" s="924"/>
+      <c r="K57" s="924"/>
       <c r="M57" s="91"/>
       <c r="N57" s="4"/>
       <c r="O57" s="4"/>
@@ -49803,19 +49803,19 @@
       <c r="W59" s="4"/>
     </row>
     <row r="60" spans="1:24" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A60" s="949" t="s">
+      <c r="A60" s="930" t="s">
         <v>122</v>
       </c>
-      <c r="B60" s="949"/>
-      <c r="C60" s="949"/>
-      <c r="D60" s="949"/>
-      <c r="E60" s="949"/>
-      <c r="F60" s="949"/>
-      <c r="G60" s="949"/>
-      <c r="H60" s="949"/>
-      <c r="I60" s="949"/>
-      <c r="J60" s="949"/>
-      <c r="K60" s="949"/>
+      <c r="B60" s="930"/>
+      <c r="C60" s="930"/>
+      <c r="D60" s="930"/>
+      <c r="E60" s="930"/>
+      <c r="F60" s="930"/>
+      <c r="G60" s="930"/>
+      <c r="H60" s="930"/>
+      <c r="I60" s="930"/>
+      <c r="J60" s="930"/>
+      <c r="K60" s="930"/>
       <c r="M60" s="91"/>
       <c r="N60" s="4"/>
       <c r="O60" s="4"/>
@@ -49836,12 +49836,12 @@
       <c r="E61" s="1"/>
       <c r="F61" s="1"/>
       <c r="G61" s="1"/>
-      <c r="H61" s="938" t="s">
+      <c r="H61" s="919" t="s">
         <v>123</v>
       </c>
-      <c r="I61" s="938"/>
-      <c r="J61" s="938"/>
-      <c r="K61" s="938"/>
+      <c r="I61" s="919"/>
+      <c r="J61" s="919"/>
+      <c r="K61" s="919"/>
       <c r="M61" s="91"/>
       <c r="N61" s="4"/>
       <c r="O61" s="4"/>
@@ -50190,6 +50190,20 @@
     <protectedRange sqref="C9:C10" name="Rango3_3_1_1_1_1_1_2_1"/>
   </protectedRanges>
   <mergeCells count="30">
+    <mergeCell ref="Z19:Z20"/>
+    <mergeCell ref="AA19:AA20"/>
+    <mergeCell ref="W19:W20"/>
+    <mergeCell ref="A5:K5"/>
+    <mergeCell ref="M31:P31"/>
+    <mergeCell ref="I31:J31"/>
+    <mergeCell ref="I30:J30"/>
+    <mergeCell ref="A17:I17"/>
+    <mergeCell ref="A6:K6"/>
+    <mergeCell ref="A14:K14"/>
+    <mergeCell ref="T9:U9"/>
+    <mergeCell ref="G23:G24"/>
+    <mergeCell ref="M30:P30"/>
+    <mergeCell ref="A15:K15"/>
     <mergeCell ref="H61:K61"/>
     <mergeCell ref="U19:V19"/>
     <mergeCell ref="X19:X20"/>
@@ -50206,20 +50220,6 @@
     <mergeCell ref="D23:D24"/>
     <mergeCell ref="E23:E24"/>
     <mergeCell ref="F23:F24"/>
-    <mergeCell ref="Z19:Z20"/>
-    <mergeCell ref="AA19:AA20"/>
-    <mergeCell ref="W19:W20"/>
-    <mergeCell ref="A5:K5"/>
-    <mergeCell ref="M31:P31"/>
-    <mergeCell ref="I31:J31"/>
-    <mergeCell ref="I30:J30"/>
-    <mergeCell ref="A17:I17"/>
-    <mergeCell ref="A6:K6"/>
-    <mergeCell ref="A14:K14"/>
-    <mergeCell ref="T9:U9"/>
-    <mergeCell ref="G23:G24"/>
-    <mergeCell ref="M30:P30"/>
-    <mergeCell ref="A15:K15"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0" right="0" top="0.59055118110236227" bottom="0" header="0.11811023622047245" footer="0"/>
@@ -50340,35 +50340,35 @@
       <c r="X6" s="178"/>
     </row>
     <row r="7" spans="1:24" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="920" t="s">
+      <c r="A7" s="932" t="s">
         <v>2</v>
       </c>
-      <c r="B7" s="920"/>
-      <c r="C7" s="920"/>
-      <c r="D7" s="920"/>
-      <c r="E7" s="920"/>
-      <c r="F7" s="920"/>
-      <c r="G7" s="920"/>
-      <c r="H7" s="920"/>
-      <c r="I7" s="920"/>
-      <c r="J7" s="920"/>
-      <c r="K7" s="920"/>
+      <c r="B7" s="932"/>
+      <c r="C7" s="932"/>
+      <c r="D7" s="932"/>
+      <c r="E7" s="932"/>
+      <c r="F7" s="932"/>
+      <c r="G7" s="932"/>
+      <c r="H7" s="932"/>
+      <c r="I7" s="932"/>
+      <c r="J7" s="932"/>
+      <c r="K7" s="932"/>
       <c r="X7" s="178"/>
     </row>
     <row r="8" spans="1:24" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="956">
+      <c r="A8" s="959">
         <v>1</v>
       </c>
-      <c r="B8" s="956"/>
-      <c r="C8" s="956"/>
-      <c r="D8" s="956"/>
-      <c r="E8" s="956"/>
-      <c r="F8" s="956"/>
-      <c r="G8" s="956"/>
-      <c r="H8" s="956"/>
-      <c r="I8" s="956"/>
-      <c r="J8" s="956"/>
-      <c r="K8" s="956"/>
+      <c r="B8" s="959"/>
+      <c r="C8" s="959"/>
+      <c r="D8" s="959"/>
+      <c r="E8" s="959"/>
+      <c r="F8" s="959"/>
+      <c r="G8" s="959"/>
+      <c r="H8" s="959"/>
+      <c r="I8" s="959"/>
+      <c r="J8" s="959"/>
+      <c r="K8" s="959"/>
       <c r="X8" s="178"/>
     </row>
     <row r="9" spans="1:24" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -50444,15 +50444,15 @@
       <c r="K13" s="308">
         <v>43845</v>
       </c>
-      <c r="M13" s="939" t="s">
+      <c r="M13" s="920" t="s">
         <v>9</v>
       </c>
-      <c r="N13" s="940"/>
-      <c r="O13" s="959" t="s">
+      <c r="N13" s="921"/>
+      <c r="O13" s="952" t="s">
         <v>69</v>
       </c>
-      <c r="P13" s="960"/>
-      <c r="Q13" s="961"/>
+      <c r="P13" s="953"/>
+      <c r="Q13" s="954"/>
       <c r="W13" s="178"/>
       <c r="X13" s="178"/>
     </row>
@@ -50476,26 +50476,26 @@
       <c r="N14" s="187" t="s">
         <v>12</v>
       </c>
-      <c r="O14" s="962"/>
-      <c r="P14" s="963"/>
-      <c r="Q14" s="964"/>
+      <c r="O14" s="955"/>
+      <c r="P14" s="956"/>
+      <c r="Q14" s="957"/>
       <c r="W14" s="178"/>
       <c r="X14" s="178"/>
     </row>
     <row r="15" spans="1:24" ht="15.6" x14ac:dyDescent="0.25">
-      <c r="A15" s="928" t="s">
+      <c r="A15" s="940" t="s">
         <v>128</v>
       </c>
-      <c r="B15" s="929"/>
-      <c r="C15" s="929"/>
-      <c r="D15" s="929"/>
-      <c r="E15" s="929"/>
-      <c r="F15" s="929"/>
-      <c r="G15" s="929"/>
-      <c r="H15" s="929"/>
-      <c r="I15" s="929"/>
-      <c r="J15" s="929"/>
-      <c r="K15" s="930"/>
+      <c r="B15" s="941"/>
+      <c r="C15" s="941"/>
+      <c r="D15" s="941"/>
+      <c r="E15" s="941"/>
+      <c r="F15" s="941"/>
+      <c r="G15" s="941"/>
+      <c r="H15" s="941"/>
+      <c r="I15" s="941"/>
+      <c r="J15" s="941"/>
+      <c r="K15" s="942"/>
       <c r="M15" s="77" t="s">
         <v>19</v>
       </c>
@@ -50509,19 +50509,19 @@
       <c r="X15" s="178"/>
     </row>
     <row r="16" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A16" s="935" t="s">
+      <c r="A16" s="947" t="s">
         <v>131</v>
       </c>
-      <c r="B16" s="936"/>
-      <c r="C16" s="936"/>
-      <c r="D16" s="936"/>
-      <c r="E16" s="936"/>
-      <c r="F16" s="936"/>
-      <c r="G16" s="936"/>
-      <c r="H16" s="936"/>
-      <c r="I16" s="936"/>
-      <c r="J16" s="936"/>
-      <c r="K16" s="937"/>
+      <c r="B16" s="948"/>
+      <c r="C16" s="948"/>
+      <c r="D16" s="948"/>
+      <c r="E16" s="948"/>
+      <c r="F16" s="948"/>
+      <c r="G16" s="948"/>
+      <c r="H16" s="948"/>
+      <c r="I16" s="948"/>
+      <c r="J16" s="948"/>
+      <c r="K16" s="949"/>
       <c r="L16" s="18"/>
       <c r="M16" s="77" t="s">
         <v>20</v>
@@ -50560,17 +50560,17 @@
       <c r="X17" s="178"/>
     </row>
     <row r="18" spans="1:24" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="925" t="s">
+      <c r="A18" s="937" t="s">
         <v>5</v>
       </c>
-      <c r="B18" s="926"/>
-      <c r="C18" s="926"/>
-      <c r="D18" s="926"/>
-      <c r="E18" s="926"/>
-      <c r="F18" s="926"/>
-      <c r="G18" s="926"/>
-      <c r="H18" s="926"/>
-      <c r="I18" s="926"/>
+      <c r="B18" s="938"/>
+      <c r="C18" s="938"/>
+      <c r="D18" s="938"/>
+      <c r="E18" s="938"/>
+      <c r="F18" s="938"/>
+      <c r="G18" s="938"/>
+      <c r="H18" s="938"/>
+      <c r="I18" s="938"/>
       <c r="J18" s="291"/>
       <c r="K18" s="292"/>
       <c r="M18" s="77">
@@ -50719,15 +50719,15 @@
       <c r="I24" s="18"/>
       <c r="J24" s="18"/>
       <c r="K24" s="144"/>
-      <c r="M24" s="939" t="s">
+      <c r="M24" s="920" t="s">
         <v>71</v>
       </c>
-      <c r="N24" s="940"/>
+      <c r="N24" s="921"/>
       <c r="O24" s="294"/>
-      <c r="P24" s="957">
+      <c r="P24" s="950">
         <v>762</v>
       </c>
-      <c r="Q24" s="958"/>
+      <c r="Q24" s="951"/>
       <c r="R24" s="202"/>
       <c r="S24" s="202"/>
       <c r="V24" s="201"/>
@@ -50736,33 +50736,33 @@
     </row>
     <row r="25" spans="1:24" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="20"/>
-      <c r="B25" s="939" t="s">
+      <c r="B25" s="920" t="s">
         <v>9</v>
       </c>
-      <c r="C25" s="940"/>
-      <c r="D25" s="833" t="s">
+      <c r="C25" s="921"/>
+      <c r="D25" s="843" t="s">
         <v>45</v>
       </c>
-      <c r="E25" s="833" t="s">
+      <c r="E25" s="843" t="s">
         <v>41</v>
       </c>
-      <c r="F25" s="833" t="s">
+      <c r="F25" s="843" t="s">
         <v>42</v>
       </c>
-      <c r="G25" s="833" t="s">
+      <c r="G25" s="843" t="s">
         <v>43</v>
       </c>
       <c r="H25" s="209"/>
-      <c r="I25" s="944" t="s">
+      <c r="I25" s="925" t="s">
         <v>36</v>
       </c>
-      <c r="J25" s="945"/>
+      <c r="J25" s="926"/>
       <c r="K25" s="144"/>
       <c r="M25" s="210" t="s">
         <v>9</v>
       </c>
       <c r="N25" s="211"/>
-      <c r="O25" s="919" t="s">
+      <c r="O25" s="931" t="s">
         <v>100</v>
       </c>
       <c r="P25" s="212" t="s">
@@ -50789,16 +50789,16 @@
       <c r="C26" s="187" t="s">
         <v>12</v>
       </c>
-      <c r="D26" s="834"/>
-      <c r="E26" s="834"/>
-      <c r="F26" s="834"/>
-      <c r="G26" s="834"/>
+      <c r="D26" s="844"/>
+      <c r="E26" s="844"/>
+      <c r="F26" s="844"/>
+      <c r="G26" s="844"/>
       <c r="H26" s="209"/>
-      <c r="I26" s="947">
+      <c r="I26" s="928">
         <f>+P24</f>
         <v>762</v>
       </c>
-      <c r="J26" s="948"/>
+      <c r="J26" s="929"/>
       <c r="K26" s="144"/>
       <c r="M26" s="213" t="s">
         <v>11</v>
@@ -50806,7 +50806,7 @@
       <c r="N26" s="187" t="s">
         <v>12</v>
       </c>
-      <c r="O26" s="919"/>
+      <c r="O26" s="931"/>
       <c r="P26" s="187" t="s">
         <v>28</v>
       </c>
@@ -50906,10 +50906,10 @@
         <v>#REF!</v>
       </c>
       <c r="H28" s="218"/>
-      <c r="I28" s="951" t="s">
+      <c r="I28" s="961" t="s">
         <v>37</v>
       </c>
-      <c r="J28" s="952"/>
+      <c r="J28" s="962"/>
       <c r="K28" s="144"/>
       <c r="M28" s="220" t="s">
         <v>31</v>
@@ -50965,11 +50965,11 @@
         <v>#REF!</v>
       </c>
       <c r="H29" s="218"/>
-      <c r="I29" s="953" t="e">
+      <c r="I29" s="963" t="e">
         <f>(R30+R32+R34+R36+R37+R39+R40+R42+R43)/100</f>
         <v>#REF!</v>
       </c>
-      <c r="J29" s="954"/>
+      <c r="J29" s="964"/>
       <c r="K29" s="144"/>
       <c r="M29" s="220" t="s">
         <v>15</v>
@@ -51085,8 +51085,8 @@
         <v>#REF!</v>
       </c>
       <c r="H31" s="218"/>
-      <c r="I31" s="924"/>
-      <c r="J31" s="924"/>
+      <c r="I31" s="936"/>
+      <c r="J31" s="936"/>
       <c r="K31" s="144"/>
       <c r="L31" s="19"/>
       <c r="M31" s="220" t="s">
@@ -51143,8 +51143,8 @@
         <v>#REF!</v>
       </c>
       <c r="H32" s="218"/>
-      <c r="I32" s="924"/>
-      <c r="J32" s="924"/>
+      <c r="I32" s="936"/>
+      <c r="J32" s="936"/>
       <c r="K32" s="144"/>
       <c r="L32" s="19"/>
       <c r="M32" s="220" t="s">
@@ -51201,8 +51201,8 @@
         <v>#REF!</v>
       </c>
       <c r="H33" s="218"/>
-      <c r="I33" s="955"/>
-      <c r="J33" s="955"/>
+      <c r="I33" s="958"/>
+      <c r="J33" s="958"/>
       <c r="K33" s="144"/>
       <c r="L33" s="19"/>
       <c r="M33" s="220" t="s">
@@ -52020,10 +52020,10 @@
       <c r="W54" s="275" t="s">
         <v>105</v>
       </c>
-      <c r="X54" s="931">
+      <c r="X54" s="943">
         <v>44090</v>
       </c>
-      <c r="Y54" s="931"/>
+      <c r="Y54" s="943"/>
       <c r="Z54" s="276"/>
       <c r="AA54" s="277"/>
       <c r="AB54" s="276"/>
@@ -52052,19 +52052,19 @@
       <c r="X57" s="178"/>
     </row>
     <row r="58" spans="1:33" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A58" s="950" t="s">
+      <c r="A58" s="960" t="s">
         <v>120</v>
       </c>
-      <c r="B58" s="950"/>
-      <c r="C58" s="950"/>
-      <c r="D58" s="950"/>
-      <c r="E58" s="950"/>
-      <c r="F58" s="950"/>
-      <c r="G58" s="950"/>
-      <c r="H58" s="950"/>
-      <c r="I58" s="950"/>
-      <c r="J58" s="950"/>
-      <c r="K58" s="950"/>
+      <c r="B58" s="960"/>
+      <c r="C58" s="960"/>
+      <c r="D58" s="960"/>
+      <c r="E58" s="960"/>
+      <c r="F58" s="960"/>
+      <c r="G58" s="960"/>
+      <c r="H58" s="960"/>
+      <c r="I58" s="960"/>
+      <c r="J58" s="960"/>
+      <c r="K58" s="960"/>
     </row>
     <row r="59" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A59" s="310" t="s">
@@ -52082,19 +52082,19 @@
       <c r="K59" s="311"/>
     </row>
     <row r="60" spans="1:33" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A60" s="950" t="s">
+      <c r="A60" s="960" t="s">
         <v>122</v>
       </c>
-      <c r="B60" s="950"/>
-      <c r="C60" s="950"/>
-      <c r="D60" s="950"/>
-      <c r="E60" s="950"/>
-      <c r="F60" s="950"/>
-      <c r="G60" s="950"/>
-      <c r="H60" s="950"/>
-      <c r="I60" s="950"/>
-      <c r="J60" s="950"/>
-      <c r="K60" s="950"/>
+      <c r="B60" s="960"/>
+      <c r="C60" s="960"/>
+      <c r="D60" s="960"/>
+      <c r="E60" s="960"/>
+      <c r="F60" s="960"/>
+      <c r="G60" s="960"/>
+      <c r="H60" s="960"/>
+      <c r="I60" s="960"/>
+      <c r="J60" s="960"/>
+      <c r="K60" s="960"/>
     </row>
     <row r="63" spans="1:33" x14ac:dyDescent="0.25">
       <c r="B63" s="5"/>
@@ -52128,6 +52128,21 @@
     <protectedRange sqref="B10:B11" name="Rango3_3_1_1_1_1_1_2_1"/>
   </protectedRanges>
   <mergeCells count="25">
+    <mergeCell ref="X54:Y54"/>
+    <mergeCell ref="O25:O26"/>
+    <mergeCell ref="A60:K60"/>
+    <mergeCell ref="I28:J28"/>
+    <mergeCell ref="I26:J26"/>
+    <mergeCell ref="I29:J29"/>
+    <mergeCell ref="I25:J25"/>
+    <mergeCell ref="A58:K58"/>
+    <mergeCell ref="I31:J31"/>
+    <mergeCell ref="A7:K7"/>
+    <mergeCell ref="I32:J32"/>
+    <mergeCell ref="I33:J33"/>
+    <mergeCell ref="A16:K16"/>
+    <mergeCell ref="A8:K8"/>
+    <mergeCell ref="A18:I18"/>
     <mergeCell ref="M24:N24"/>
     <mergeCell ref="P24:Q24"/>
     <mergeCell ref="F25:F26"/>
@@ -52138,21 +52153,6 @@
     <mergeCell ref="B25:C25"/>
     <mergeCell ref="D25:D26"/>
     <mergeCell ref="E25:E26"/>
-    <mergeCell ref="A7:K7"/>
-    <mergeCell ref="I32:J32"/>
-    <mergeCell ref="I33:J33"/>
-    <mergeCell ref="A16:K16"/>
-    <mergeCell ref="A8:K8"/>
-    <mergeCell ref="A18:I18"/>
-    <mergeCell ref="X54:Y54"/>
-    <mergeCell ref="O25:O26"/>
-    <mergeCell ref="A60:K60"/>
-    <mergeCell ref="I28:J28"/>
-    <mergeCell ref="I26:J26"/>
-    <mergeCell ref="I29:J29"/>
-    <mergeCell ref="I25:J25"/>
-    <mergeCell ref="A58:K58"/>
-    <mergeCell ref="I31:J31"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0" right="0" top="0.39370078740157483" bottom="0" header="0.11811023622047245" footer="0"/>
@@ -52235,35 +52235,35 @@
       <c r="H4" s="177"/>
     </row>
     <row r="5" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="920" t="s">
+      <c r="A5" s="932" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="920"/>
-      <c r="C5" s="920"/>
-      <c r="D5" s="920"/>
-      <c r="E5" s="920"/>
-      <c r="F5" s="920"/>
-      <c r="G5" s="920"/>
-      <c r="H5" s="920"/>
-      <c r="I5" s="920"/>
-      <c r="J5" s="920"/>
-      <c r="K5" s="920"/>
+      <c r="B5" s="932"/>
+      <c r="C5" s="932"/>
+      <c r="D5" s="932"/>
+      <c r="E5" s="932"/>
+      <c r="F5" s="932"/>
+      <c r="G5" s="932"/>
+      <c r="H5" s="932"/>
+      <c r="I5" s="932"/>
+      <c r="J5" s="932"/>
+      <c r="K5" s="932"/>
     </row>
     <row r="6" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="927">
+      <c r="A6" s="939">
         <f>+K12</f>
         <v>44</v>
       </c>
-      <c r="B6" s="927"/>
-      <c r="C6" s="927"/>
-      <c r="D6" s="927"/>
-      <c r="E6" s="927"/>
-      <c r="F6" s="927"/>
-      <c r="G6" s="927"/>
-      <c r="H6" s="927"/>
-      <c r="I6" s="927"/>
-      <c r="J6" s="927"/>
-      <c r="K6" s="927"/>
+      <c r="B6" s="939"/>
+      <c r="C6" s="939"/>
+      <c r="D6" s="939"/>
+      <c r="E6" s="939"/>
+      <c r="F6" s="939"/>
+      <c r="G6" s="939"/>
+      <c r="H6" s="939"/>
+      <c r="I6" s="939"/>
+      <c r="J6" s="939"/>
+      <c r="K6" s="939"/>
       <c r="Q6" s="259" t="s">
         <v>101</v>
       </c>
@@ -52329,10 +52329,10 @@
       <c r="Q9" s="275" t="s">
         <v>105</v>
       </c>
-      <c r="R9" s="931">
+      <c r="R9" s="943">
         <v>44090</v>
       </c>
-      <c r="S9" s="931"/>
+      <c r="S9" s="943"/>
       <c r="T9" s="276"/>
       <c r="U9" s="277"/>
       <c r="V9" s="276"/>
@@ -52413,37 +52413,37 @@
       <c r="U13" s="3"/>
     </row>
     <row r="14" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="928" t="s">
+      <c r="A14" s="940" t="s">
         <v>128</v>
       </c>
-      <c r="B14" s="929"/>
-      <c r="C14" s="929"/>
-      <c r="D14" s="929"/>
-      <c r="E14" s="929"/>
-      <c r="F14" s="929"/>
-      <c r="G14" s="929"/>
-      <c r="H14" s="929"/>
-      <c r="I14" s="929"/>
-      <c r="J14" s="929"/>
-      <c r="K14" s="930"/>
+      <c r="B14" s="941"/>
+      <c r="C14" s="941"/>
+      <c r="D14" s="941"/>
+      <c r="E14" s="941"/>
+      <c r="F14" s="941"/>
+      <c r="G14" s="941"/>
+      <c r="H14" s="941"/>
+      <c r="I14" s="941"/>
+      <c r="J14" s="941"/>
+      <c r="K14" s="942"/>
       <c r="S14" s="5"/>
       <c r="T14" s="5"/>
       <c r="U14" s="70"/>
     </row>
     <row r="15" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="935" t="s">
+      <c r="A15" s="947" t="s">
         <v>131</v>
       </c>
-      <c r="B15" s="936"/>
-      <c r="C15" s="936"/>
-      <c r="D15" s="936"/>
-      <c r="E15" s="936"/>
-      <c r="F15" s="936"/>
-      <c r="G15" s="936"/>
-      <c r="H15" s="936"/>
-      <c r="I15" s="936"/>
-      <c r="J15" s="936"/>
-      <c r="K15" s="937"/>
+      <c r="B15" s="948"/>
+      <c r="C15" s="948"/>
+      <c r="D15" s="948"/>
+      <c r="E15" s="948"/>
+      <c r="F15" s="948"/>
+      <c r="G15" s="948"/>
+      <c r="H15" s="948"/>
+      <c r="I15" s="948"/>
+      <c r="J15" s="948"/>
+      <c r="K15" s="949"/>
       <c r="S15" s="5"/>
       <c r="T15" s="5"/>
       <c r="U15" s="71"/>
@@ -52465,17 +52465,17 @@
       <c r="U16" s="70"/>
     </row>
     <row r="17" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="925" t="s">
+      <c r="A17" s="937" t="s">
         <v>5</v>
       </c>
-      <c r="B17" s="926"/>
-      <c r="C17" s="926"/>
-      <c r="D17" s="926"/>
-      <c r="E17" s="926"/>
-      <c r="F17" s="926"/>
-      <c r="G17" s="926"/>
-      <c r="H17" s="926"/>
-      <c r="I17" s="926"/>
+      <c r="B17" s="938"/>
+      <c r="C17" s="938"/>
+      <c r="D17" s="938"/>
+      <c r="E17" s="938"/>
+      <c r="F17" s="938"/>
+      <c r="G17" s="938"/>
+      <c r="H17" s="938"/>
+      <c r="I17" s="938"/>
       <c r="J17" s="291" t="s">
         <v>124</v>
       </c>
@@ -52571,16 +52571,16 @@
       <c r="I22" s="242"/>
       <c r="J22" s="18"/>
       <c r="K22" s="243"/>
-      <c r="M22" s="967" t="s">
+      <c r="M22" s="965" t="s">
         <v>71</v>
       </c>
-      <c r="N22" s="968"/>
+      <c r="N22" s="966"/>
       <c r="O22" s="280"/>
-      <c r="P22" s="969">
+      <c r="P22" s="967">
         <f>SUM(O25:O42)</f>
         <v>9543.9950657520003</v>
       </c>
-      <c r="Q22" s="958"/>
+      <c r="Q22" s="951"/>
       <c r="R22" s="77" t="s">
         <v>73</v>
       </c>
@@ -52595,33 +52595,33 @@
     </row>
     <row r="23" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="20"/>
-      <c r="B23" s="965" t="s">
+      <c r="B23" s="973" t="s">
         <v>9</v>
       </c>
-      <c r="C23" s="965"/>
-      <c r="D23" s="966" t="s">
+      <c r="C23" s="973"/>
+      <c r="D23" s="970" t="s">
         <v>45</v>
       </c>
-      <c r="E23" s="966" t="s">
+      <c r="E23" s="970" t="s">
         <v>41</v>
       </c>
-      <c r="F23" s="966" t="s">
+      <c r="F23" s="970" t="s">
         <v>42</v>
       </c>
-      <c r="G23" s="966" t="s">
+      <c r="G23" s="970" t="s">
         <v>43</v>
       </c>
       <c r="H23" s="18"/>
-      <c r="I23" s="944" t="s">
+      <c r="I23" s="925" t="s">
         <v>36</v>
       </c>
-      <c r="J23" s="945"/>
+      <c r="J23" s="926"/>
       <c r="K23" s="144"/>
       <c r="M23" s="67" t="s">
         <v>9</v>
       </c>
       <c r="N23" s="68"/>
-      <c r="O23" s="919" t="s">
+      <c r="O23" s="931" t="s">
         <v>100</v>
       </c>
       <c r="P23" s="9" t="s">
@@ -52652,16 +52652,16 @@
       <c r="C24" s="244" t="s">
         <v>12</v>
       </c>
-      <c r="D24" s="966"/>
-      <c r="E24" s="966"/>
-      <c r="F24" s="966"/>
-      <c r="G24" s="966"/>
+      <c r="D24" s="970"/>
+      <c r="E24" s="970"/>
+      <c r="F24" s="970"/>
+      <c r="G24" s="970"/>
       <c r="H24" s="245"/>
-      <c r="I24" s="947">
+      <c r="I24" s="928">
         <f>+P22</f>
         <v>9543.9950657520003</v>
       </c>
-      <c r="J24" s="948"/>
+      <c r="J24" s="929"/>
       <c r="K24" s="144"/>
       <c r="M24" s="65" t="s">
         <v>11</v>
@@ -52669,7 +52669,7 @@
       <c r="N24" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="O24" s="919"/>
+      <c r="O24" s="931"/>
       <c r="P24" s="10" t="s">
         <v>28</v>
       </c>
@@ -52790,10 +52790,10 @@
         <v>100</v>
       </c>
       <c r="H26" s="245"/>
-      <c r="I26" s="951" t="s">
+      <c r="I26" s="961" t="s">
         <v>37</v>
       </c>
-      <c r="J26" s="952"/>
+      <c r="J26" s="962"/>
       <c r="K26" s="144"/>
       <c r="M26" s="74">
         <v>2.5</v>
@@ -52870,11 +52870,11 @@
         <v>100</v>
       </c>
       <c r="H27" s="245"/>
-      <c r="I27" s="972">
+      <c r="I27" s="971">
         <f>(R28+R30+R32+R34+R35+R37+R38+R40+R41)/100</f>
         <v>6.8505867560771163</v>
       </c>
-      <c r="J27" s="973"/>
+      <c r="J27" s="972"/>
       <c r="K27" s="144"/>
       <c r="M27" s="74">
         <v>2</v>
@@ -53029,10 +53029,10 @@
         <v>98.973176865046099</v>
       </c>
       <c r="H29" s="245"/>
-      <c r="I29" s="951" t="s">
+      <c r="I29" s="961" t="s">
         <v>65</v>
       </c>
-      <c r="J29" s="952"/>
+      <c r="J29" s="962"/>
       <c r="K29" s="144"/>
       <c r="L29" s="19"/>
       <c r="M29" s="74">
@@ -53110,11 +53110,11 @@
         <v>44.991617770326911</v>
       </c>
       <c r="H30" s="245"/>
-      <c r="I30" s="970">
+      <c r="I30" s="968">
         <f>+Z38</f>
         <v>0.5</v>
       </c>
-      <c r="J30" s="971"/>
+      <c r="J30" s="969"/>
       <c r="K30" s="144"/>
       <c r="L30" s="19"/>
       <c r="M30" s="74">
@@ -53271,8 +53271,8 @@
         <v>0.20955574182733017</v>
       </c>
       <c r="H32" s="245"/>
-      <c r="I32" s="924"/>
-      <c r="J32" s="924"/>
+      <c r="I32" s="936"/>
+      <c r="J32" s="936"/>
       <c r="K32" s="144"/>
       <c r="L32" s="19"/>
       <c r="M32" s="74">
@@ -53350,8 +53350,8 @@
         <v>0</v>
       </c>
       <c r="H33" s="245"/>
-      <c r="I33" s="924"/>
-      <c r="J33" s="924"/>
+      <c r="I33" s="936"/>
+      <c r="J33" s="936"/>
       <c r="K33" s="144"/>
       <c r="L33" s="19"/>
       <c r="M33" s="74">
@@ -53424,8 +53424,8 @@
       </c>
       <c r="G34" s="303"/>
       <c r="H34" s="245"/>
-      <c r="I34" s="955"/>
-      <c r="J34" s="955"/>
+      <c r="I34" s="958"/>
+      <c r="J34" s="958"/>
       <c r="K34" s="144"/>
       <c r="L34" s="19"/>
       <c r="M34" s="23" t="s">
@@ -54073,27 +54073,27 @@
       <c r="K54" s="297"/>
     </row>
     <row r="55" spans="1:21" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A55" s="949" t="s">
+      <c r="A55" s="930" t="s">
         <v>122</v>
       </c>
-      <c r="B55" s="949"/>
-      <c r="C55" s="949"/>
-      <c r="D55" s="949"/>
-      <c r="E55" s="949"/>
-      <c r="F55" s="949"/>
-      <c r="G55" s="949"/>
-      <c r="H55" s="949"/>
-      <c r="I55" s="949"/>
-      <c r="J55" s="949"/>
-      <c r="K55" s="949"/>
+      <c r="B55" s="930"/>
+      <c r="C55" s="930"/>
+      <c r="D55" s="930"/>
+      <c r="E55" s="930"/>
+      <c r="F55" s="930"/>
+      <c r="G55" s="930"/>
+      <c r="H55" s="930"/>
+      <c r="I55" s="930"/>
+      <c r="J55" s="930"/>
+      <c r="K55" s="930"/>
     </row>
     <row r="56" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="H56" s="938" t="s">
+      <c r="H56" s="919" t="s">
         <v>123</v>
       </c>
-      <c r="I56" s="938"/>
-      <c r="J56" s="938"/>
-      <c r="K56" s="938"/>
+      <c r="I56" s="919"/>
+      <c r="J56" s="919"/>
+      <c r="K56" s="919"/>
     </row>
   </sheetData>
   <protectedRanges>
@@ -54103,6 +54103,15 @@
     <protectedRange sqref="B9:B10" name="Rango3_3_1_1_1_1_1_2_1"/>
   </protectedRanges>
   <mergeCells count="25">
+    <mergeCell ref="B23:C23"/>
+    <mergeCell ref="D23:D24"/>
+    <mergeCell ref="E23:E24"/>
+    <mergeCell ref="A5:K5"/>
+    <mergeCell ref="A6:K6"/>
+    <mergeCell ref="A14:K14"/>
+    <mergeCell ref="A15:K15"/>
+    <mergeCell ref="I23:J23"/>
+    <mergeCell ref="G23:G24"/>
     <mergeCell ref="A55:K55"/>
     <mergeCell ref="H56:K56"/>
     <mergeCell ref="O23:O24"/>
@@ -54119,15 +54128,6 @@
     <mergeCell ref="I26:J26"/>
     <mergeCell ref="I24:J24"/>
     <mergeCell ref="I27:J27"/>
-    <mergeCell ref="B23:C23"/>
-    <mergeCell ref="D23:D24"/>
-    <mergeCell ref="E23:E24"/>
-    <mergeCell ref="A5:K5"/>
-    <mergeCell ref="A6:K6"/>
-    <mergeCell ref="A14:K14"/>
-    <mergeCell ref="A15:K15"/>
-    <mergeCell ref="I23:J23"/>
-    <mergeCell ref="G23:G24"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0" right="0" top="0.59055118110236227" bottom="0" header="0.11811023622047245" footer="0"/>

</xml_diff>